<commit_message>
Add Phase C's style and contest rows to the spreadsheet — snapshot unmoved
GDD_V3 §5.1's three styles as one row each (early top-speed multiplier, fade start shift, fade
penalty multiplier, and whether the style contests the lead), the early window, §5.2's expression
band U(0.30, 1.30), and §5.3's contest rule (window, 2 m, +3%, 0.05). All ⚖️ estimates from the GDD.

Written by the new packages/engine/scripts/add-phase-c-rows.ts, a copy of Phase B's upserter; the
workbook was re-checked for formula cells (none) and cell styles (one cellXf, the default) first.
balance.json regenerated with `npm run balance`. Nothing reads the new keys yet, so the golden
snapshot does not move.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JijDDeDKx6mZGhfWE6YEK7
</commit_message>
<xml_diff>
--- a/design/space_dog_racing_economy.xlsx
+++ b/design/space_dog_racing_economy.xlsx
@@ -526,7 +526,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D159"/>
+  <dimension ref="A1:D182"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1763,9 +1763,204 @@
         <v>1.55</v>
       </c>
     </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>Running styles (GDD_V3 §5.1–5.2 — a redistribution of the same energy, not a bonus)</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>Front-runner: early top-speed multiplier</v>
+      </c>
+      <c r="B162">
+        <v>1.08</v>
+      </c>
+      <c r="C162" t="str">
+        <v>Bursts from the boxes, leads early, pays for it later. Leans on Acceleration</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>Front-runner: fade start shift</v>
+      </c>
+      <c r="B163">
+        <v>-0.12</v>
+      </c>
+      <c r="C163" t="str">
+        <v>In the same units as the fade point itself; negative is earlier</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>Front-runner: fade penalty multiplier</v>
+      </c>
+      <c r="B164">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>Front-runner: contests the lead (1 = yes)</v>
+      </c>
+      <c r="B165">
+        <v>1</v>
+      </c>
+      <c r="C165" t="str">
+        <v>Which styles the contest rule of §5.3 reads. A flag on the row, so the rule never names a style</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>Stalker: early top-speed multiplier</v>
+      </c>
+      <c r="B166">
+        <v>1</v>
+      </c>
+      <c r="C166" t="str">
+        <v>The baseline: even pace, sits handy, wins by being better. Leans on Speed</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>Stalker: fade start shift</v>
+      </c>
+      <c r="B167">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>Stalker: fade penalty multiplier</v>
+      </c>
+      <c r="B168">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>Stalker: contests the lead (1 = yes)</v>
+      </c>
+      <c r="B169">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>Closer: early top-speed multiplier</v>
+      </c>
+      <c r="B170">
+        <v>0.94</v>
+      </c>
+      <c r="C170" t="str">
+        <v>Slow away, comes home hardest. Leans on Stamina</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>Closer: fade start shift</v>
+      </c>
+      <c r="B171">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>Closer: fade penalty multiplier</v>
+      </c>
+      <c r="B172">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>Closer: contests the lead (1 = yes)</v>
+      </c>
+      <c r="B173">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>Style: the early part of the race (fraction of the trip)</v>
+      </c>
+      <c r="B174">
+        <v>0.333</v>
+      </c>
+      <c r="C174" t="str">
+        <v>Where the early top-speed multiplier applies. The first third, the same window the contest rule reads</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>Style expression: minimum</v>
+      </c>
+      <c r="B175">
+        <v>0.3</v>
+      </c>
+      <c r="C175" t="str">
+        <v>GDD_V3 §5.2, V13: one U(min, max) draw per runner per race, scaling how strongly its style applies that day. NOT a multiplier on speed — the area under the curve stays put and only its shape moves</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>Style expression: maximum</v>
+      </c>
+      <c r="B176">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>The contest rule (GDD_V3 §5.3 — a kill switch, not a tuning target)</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>Contest: window (fraction of the trip)</v>
+      </c>
+      <c r="B179">
+        <v>0.333</v>
+      </c>
+      <c r="C179" t="str">
+        <v>While a front-runner is inside the first third of the race</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>Contest: distance at the head of the field (metres)</v>
+      </c>
+      <c r="B180">
+        <v>2</v>
+      </c>
+      <c r="C180" t="str">
+        <v>…and another dog is within this of it at the head of the field</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>Contest: speed boost while contesting</v>
+      </c>
+      <c r="B181">
+        <v>0.03</v>
+      </c>
+      <c r="C181" t="str">
+        <v>…both get this much on current speed</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>Contest: fade start cost for a whole first third contested</v>
+      </c>
+      <c r="B182">
+        <v>0.05</v>
+      </c>
+      <c r="C182" t="str">
+        <v>…and their fade point moves this much earlier, in proportion to the share of the window spent contesting. A cost larger than the boost is worth. If the closer’s gap against a front-runner-heavy field is under 4 points, the rule is cut, not tuned</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D159"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D182"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add the hot pace rows to the spreadsheet — snapshot unmoved
GDD_V3 §5.3, V14, §14 Q10: the contest rule's replacement. Four cells for the rule (the window, how
close two front-runners must be at the head to light it, how close to the leader a runner must be to
pay, and what a whole window in a hot lead group costs in metres of fade point) and one per style
saying whether that style lights the pace — a style is a row, so the rule will count a flag and never
ask a style its name. Written by the new add-phase-c2-rows.ts (a copy of Phase C's upserter; the
workbook re-checked first: no formula cells, one cell style). balance.json regenerated with npm run
balance. Nothing reads the rows yet, so the golden snapshot does not move; npm test 26 green.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WunFyptq75QFsNfLSWXWKg
</commit_message>
<xml_diff>
--- a/design/space_dog_racing_economy.xlsx
+++ b/design/space_dog_racing_economy.xlsx
@@ -526,7 +526,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D192"/>
+  <dimension ref="A1:D201"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2008,9 +2008,85 @@
         <v>4</v>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>The hot pace (GDD_V3 §5.3 — two front-runners at the head light it; the lead group pays)</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>Hot pace: window (fraction of the trip)</v>
+      </c>
+      <c r="B195">
+        <v>0.333</v>
+      </c>
+      <c r="C195" t="str">
+        <v>The pace can only be hot while the leader is inside this much of the trip. The first third, as for the style curve</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>Hot pace: front-runners within this of each other at the head (metres)</v>
+      </c>
+      <c r="B196">
+        <v>2</v>
+      </c>
+      <c r="C196" t="str">
+        <v>Two or more runners whose style lights the pace, both this close to the leader (so to each other), make the pace hot. One alone never does</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>Hot pace: the lead group, within this of the leader (metres)</v>
+      </c>
+      <c r="B197">
+        <v>4</v>
+      </c>
+      <c r="C197" t="str">
+        <v>While the pace is hot, every runner this close to the leader pays — front-runners and the stalkers sitting on them alike. A dog further back pays nothing</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>Hot pace: fade point cost for a whole window in a hot lead group (metres)</v>
+      </c>
+      <c r="B198">
+        <v>30</v>
+      </c>
+      <c r="C198" t="str">
+        <v>Pro rata to the ground a dog covers in the lead group while the pace is hot. Metres, like the fade point itself (A7)</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>Front-runner: lights the pace (1 = yes)</v>
+      </c>
+      <c r="B199">
+        <v>1</v>
+      </c>
+      <c r="C199" t="str">
+        <v>A style is a row: the rule counts runners whose style says 1 here, and never asks a style its name</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>Stalker: lights the pace (1 = yes)</v>
+      </c>
+      <c r="B200">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>Closer: lights the pace (1 = yes)</v>
+      </c>
+      <c r="B201">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D192"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D201"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Phase D1's spreadsheet rows: dog offers, race-day conditions, the local runner — data only, snapshot unmoved
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NHScg2aSAAFiFAd9PYoStX
</commit_message>
<xml_diff>
--- a/design/space_dog_racing_economy.xlsx
+++ b/design/space_dog_racing_economy.xlsx
@@ -526,7 +526,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D205"/>
+  <dimension ref="A1:D225"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2114,9 +2114,163 @@
         <v>What the fade in fractions (v3b) did to the whole field before A7 made the fade metres: a time gap stays a time gap, and the metres it shows at the line shrink with the speed</v>
       </c>
     </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>Dog offers (GDD_V3 §9.2 — age, one stat, and patter that is sometimes a lie)</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>Dog offer: the seller lies, chance</v>
+      </c>
+      <c r="B208">
+        <v>0.35</v>
+      </c>
+      <c r="C208" t="str">
+        <v>Before the card row's own multiplier: a monk never lies (×0), a man in a long coat usually does. A lie is a claimed stat that is really poor</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>Dog offer: rating, mean</v>
+      </c>
+      <c r="B209">
+        <v>50</v>
+      </c>
+      <c r="C209" t="str">
+        <v>Where an offered dog's stats centre. A dealt dog rates 50, so the average offer is a sideways move and the gamble is the spread</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>Dog offer: rating, sd</v>
+      </c>
+      <c r="B210">
+        <v>7</v>
+      </c>
+      <c r="C210" t="str">
+        <v>Spread of the offered dog's level, before its shape. Rating is never shown</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>Dog offer: youngest age</v>
+      </c>
+      <c r="B211">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>Dog offer: oldest age</v>
+      </c>
+      <c r="B212">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>Dog offer: the claimed stat, when honest (points above the level)</v>
+      </c>
+      <c r="B213">
+        <v>10</v>
+      </c>
+      <c r="C213" t="str">
+        <v>The seller talks up one stat you cannot see. Honest, it really is this far above the dog's level</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>Dog offer: the claimed stat, when lying (points below the level)</v>
+      </c>
+      <c r="B214">
+        <v>12</v>
+      </c>
+      <c r="C214" t="str">
+        <v>Lying, the stat he talks up is this far below it</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>Race-day conditions (Phase D1 — drawn on arrival, applied on race day, never priced by the book)</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>Condition: a knock, chance per stable dog per weekend</v>
+      </c>
+      <c r="B217">
+        <v>0.06</v>
+      </c>
+      <c r="C217" t="str">
+        <v>Drawn for every stable dog at arrival, one draw a dog whatever it lands on, so the stream never depends on the outcome</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>Condition: a knock, fitness on race day</v>
+      </c>
+      <c r="B218">
+        <v>-30</v>
+      </c>
+      <c r="C218" t="str">
+        <v>Applied to the runner, never to the stored fitness: every screen and the whole book go on reading the dog as it was</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>Condition: off its feed, chance per stable dog per weekend</v>
+      </c>
+      <c r="B219">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>Condition: off its feed, fitness on race day</v>
+      </c>
+      <c r="B220">
+        <v>-15</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>Condition: buzzing, chance per stable dog per weekend</v>
+      </c>
+      <c r="B221">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>Condition: buzzing, speed on race day (stat points)</v>
+      </c>
+      <c r="B222">
+        <v>8</v>
+      </c>
+      <c r="C222" t="str">
+        <v>Like the lucky bone, but nobody knows unless tipped — the owner included</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>The free local runner (GDD_V3 §4.4 — a stable short of fit dogs is lent one)</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>Local runner: a dog counts as fit at this fitness or above</v>
+      </c>
+      <c r="B225">
+        <v>50</v>
+      </c>
+      <c r="C225" t="str">
+        <v>The injury-doubling line (§4.4). A stable with fewer than three uninjured dogs at or above it is lent a local for the Bronze Dash</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D205"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D225"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Retune at 800 seasons: buzzing +3 speed, dog offers centred on 42 — snapshot moves
The re-baseline read a buzzing dog at +33.4% a Bone (band +10-30%) and mean end worth at 39,908,
40,091 after a first trim — on the line of its 25-40k band, where the paired-seed noise is about
200. conditionBuzzingSpeed 5 -> 4 -> 3 and dogOfferRatingMean 44 -> 42, both in the sheet.

800 seasons all-Normal: mean end worth 39,710; a buzzing dog +20.1% a Bone, a stable dog blind
-1.3%, the house margin -12.6%, a knock -60.5%, off its feed -29.7%; tipped buzzing bets Normal
placed +33.6% (1,386 bets, mostly long prices); dog offers 0.90 a stable-season, 2.89 swings for a
stable that wants one.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NHScg2aSAAFiFAd9PYoStX
</commit_message>
<xml_diff>
--- a/design/space_dog_racing_economy.xlsx
+++ b/design/space_dog_racing_economy.xlsx
@@ -2135,10 +2135,10 @@
         <v>Dog offer: rating, mean</v>
       </c>
       <c r="B209">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C209" t="str">
-        <v>Where an offered dog's stats centre. A dealt dog rates 50, so the average offer is a step down and the gamble is the spread and the patter. 50 at first; 44 in Phase D1, because at 50 the Pound alone lifted mean end worth about 2,000 and out of its 25-40k band</v>
+        <v>Where an offered dog's stats centre. A dealt dog rates 50, so the average offer is a step down and the gamble is the spread and the patter. 50 at first; 44 in Phase D1, and then 42, because at 50 the Pound alone lifted mean end worth about 2,000 and out of its 25-40k band, and at 44 it sat on the 40k line</v>
       </c>
     </row>
     <row r="210">
@@ -2246,10 +2246,10 @@
         <v>Condition: buzzing, speed on race day (stat points)</v>
       </c>
       <c r="B222">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C222" t="str">
-        <v>Like the lucky bone, but nobody knows unless tipped — the owner included</v>
+        <v>Like the lucky bone, but nobody knows unless tipped — the owner included. 8 read +53% a Bone backed, 5 read +33% and 4 +32% at 800 seasons (the standard error is about 4 points); 3 is the setting</v>
       </c>
     </row>
     <row r="224">

</xml_diff>

<commit_message>
Spreadsheet rows for Phase D2: staff cuts and bonus sizes, the nobble, the stewards' catch and fine — snapshot unmoved
23 rows through packages/engine/scripts/add-phase-d2-rows.ts (a copy of
add-phase-d-rows.ts), then npm run balance. Data only: nothing reads them yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WsLDGbvja34vpn67tEoxoe
</commit_message>
<xml_diff>
--- a/design/space_dog_racing_economy.xlsx
+++ b/design/space_dog_racing_economy.xlsx
@@ -526,7 +526,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D225"/>
+  <dimension ref="A1:D252"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2268,9 +2268,239 @@
         <v>A stable with fewer than three uninjured dogs at or above this is lent a local for the Bronze Dash (§4.4). Tried at 50, the injury-doubling line: Normal's race-rest rhythm puts a dog under 50 most weeks, so half of all weekends lent a runner (4.8 a stable-season) and it was a purse, not a guard. At 30: 1.2 a stable-season</v>
       </c>
     </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>Staff (GDD_V3 §8 — two trainers, paid a cut of race prize money only)</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>Staff: trainers dealt to each stable at the start of a game</v>
+      </c>
+      <c r="B228">
+        <v>2</v>
+      </c>
+      <c r="C228" t="str">
+        <v>Two slots, everyone a trainer (§8.1). Dealt at createSeason from the staff rows; the only way to change one in Phase D is a Bar card</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>Staff cut: +1 stat a week</v>
+      </c>
+      <c r="B229">
+        <v>0.03</v>
+      </c>
+      <c r="C229" t="str">
+        <v>Commission, a share of race prize money only (§8.1). A trainer with one bonus takes its cut; with two, the sum plus the premium below, capped</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>Staff cut: +5 fitness recovery a week</v>
+      </c>
+      <c r="B230">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>Staff cut: injury chance halved</v>
+      </c>
+      <c r="B231">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>Staff cut: injury duration −1 week</v>
+      </c>
+      <c r="B232">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>Staff cut: reveals a rival dog's style a week</v>
+      </c>
+      <c r="B233">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>Staff cut: next planet's band position for all six goods</v>
+      </c>
+      <c r="B234">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>Staff cut: +10% prize money</v>
+      </c>
+      <c r="B235">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>Staff cut: Explore less likely to go badly</v>
+      </c>
+      <c r="B236">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v>Staff cut: premium for a trainer with two bonuses</v>
+      </c>
+      <c r="B237">
+        <v>0.02</v>
+      </c>
+      <c r="C237" t="str">
+        <v>§8.2: "two of the above, 6–10%". The cheapest pair (2% + 2%) lands on 6%</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v>Staff cut: the most a trainer takes</v>
+      </c>
+      <c r="B238">
+        <v>0.1</v>
+      </c>
+      <c r="C238" t="str">
+        <v>§8.1: 1–10%. A 10% trainer on a stable earning 30,000 in purses costs 3,000</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>Staff bonus: stat points a week, to each dog</v>
+      </c>
+      <c r="B239">
+        <v>1</v>
+      </c>
+      <c r="C239" t="str">
+        <v>At the jump, beside the food, on the dog's weakest stat by the rating's weights — a rule, not a draw, so hiring a trainer never moves the game's stream</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>Staff bonus: fitness a week, to a dog that did not run</v>
+      </c>
+      <c r="B240">
+        <v>5</v>
+      </c>
+      <c r="C240" t="str">
+        <v>Folded into weeklyFitnessDelta's bonus, so it goes through the week's one clamp</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>Staff bonus: injury chance ×</v>
+      </c>
+      <c r="B241">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>Staff bonus: weeks off a layoff, at the roll</v>
+      </c>
+      <c r="B242">
+        <v>1</v>
+      </c>
+      <c r="C242" t="str">
+        <v>Never below one week</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v>Staff bonus: extra prize money, share of the purse</v>
+      </c>
+      <c r="B243">
+        <v>0.1</v>
+      </c>
+      <c r="C243" t="str">
+        <v>Added before the commission is taken</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v>Staff bonus: an Explore card's bad-outcome chance ×</v>
+      </c>
+      <c r="B244">
+        <v>0.5</v>
+      </c>
+      <c r="C244" t="str">
+        <v>Read by every card through the kit's risk() and luck() helpers, never by a branch</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v>Sabotage (GDD_V3 §9.3 — a nobble, a bought box, and the stewards who might notice)</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v>Sabotage: a nobbled runner's fitness on race day</v>
+      </c>
+      <c r="B247">
+        <v>-25</v>
+      </c>
+      <c r="C247" t="str">
+        <v>Applied to the runner, like a race-day condition: the book has struck its prices and the victim's stated fitness never changes</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>Sabotage: stewards catch a nobbler, chance (any planet without its own)</v>
+      </c>
+      <c r="B248">
+        <v>0.35</v>
+      </c>
+      <c r="C248" t="str">
+        <v>Rolled on race day from one draw per stable, made every week whether or not anybody booked a job, so the game stream never depends on a door</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>Sabotage: catch chance at Lagrange Lows</v>
+      </c>
+      <c r="B249">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>Sabotage: catch chance at Holy Bark</v>
+      </c>
+      <c r="B250">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="str">
+        <v>Sabotage: caught, a flat fine</v>
+      </c>
+      <c r="B251">
+        <v>800</v>
+      </c>
+      <c r="C251" t="str">
+        <v>Paid as far as the cash goes: nobody is pushed into debt (V10)</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="str">
+        <v>Sabotage: caught, share of what the nobbler had on the race</v>
+      </c>
+      <c r="B252">
+        <v>0.25</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D225"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D252"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Spreadsheet rows for Phase E1: game length, targets, the off-season — snapshot unmoved
add-phase-e1-rows.ts (a copy of add-phase-d2-rows.ts) adds nine rows under two new sections:
the seasons a table may choose (1-5), the suggested targets (60,000 and 150,000), the season cap
for a Target game (10), a trainer's off-season notice (15%), the retirement replacement's lie
multiplier, and the AI's two retirement thresholds (500 Bones over the cheapest dog; any dog of
6). Data only: nothing reads them yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Di3oPY6yj1QhBV6FuBjsAF
</commit_message>
<xml_diff>
--- a/design/space_dog_racing_economy.xlsx
+++ b/design/space_dog_racing_economy.xlsx
@@ -526,7 +526,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D252"/>
+  <dimension ref="A1:D265"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2507,9 +2507,109 @@
         <v>0.25</v>
       </c>
     </row>
+    <row r="254">
+      <c r="A254" t="str">
+        <v>The game (GDD_V3 §2.1 — 1 to 5 seasons, or Race to a Target)</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="str">
+        <v>Game: fewest seasons a table may choose</v>
+      </c>
+      <c r="B255">
+        <v>1</v>
+      </c>
+      <c r="C255" t="str">
+        <v>The default game is one season, and a setup that names no length means one season</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="str">
+        <v>Game: most seasons a table may choose</v>
+      </c>
+      <c r="B256">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="str">
+        <v>Target: suggested net worth, a short game</v>
+      </c>
+      <c r="B257">
+        <v>60000</v>
+      </c>
+      <c r="C257" t="str">
+        <v>Net worth is checked at the end of every weekend; the first crossing ends the game at the end of that weekend, and the highest net worth wins (§2.1)</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="str">
+        <v>Target: suggested net worth, a long game</v>
+      </c>
+      <c r="B258">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v>Target: the most seasons a Target game runs</v>
+      </c>
+      <c r="B259">
+        <v>10</v>
+      </c>
+      <c r="C259" t="str">
+        <v>A cap so a target nobody reaches still ends. If it bites, the highest net worth wins as usual</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="str">
+        <v>The off-season (GDD_V3 §2.2 — age, one retirement, the staff notice)</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="str">
+        <v>Off-season: a trainer leaves, chance each</v>
+      </c>
+      <c r="B262">
+        <v>0.15</v>
+      </c>
+      <c r="C262" t="str">
+        <v>Rolled per trainer on the stable's own off-season stream. A stable left with fewer than two is offered one candidate</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="str">
+        <v>Off-season: the replacement's seller lies, × the dog-offer rate</v>
+      </c>
+      <c r="B263">
+        <v>1</v>
+      </c>
+      <c r="C263" t="str">
+        <v>A retirement is offered a replacement under §9.2: age, one true stat, and patter that lies at this × 0.35</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>Off-season: AI retires when the offer beats its cheapest dog by (Bones)</v>
+      </c>
+      <c r="B264">
+        <v>500</v>
+      </c>
+      <c r="C264" t="str">
+        <v>Normal's rule: the offer as it can read it (estimateOffer) against the cheapest dog's book value plus this. Hard uses half</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="str">
+        <v>Off-season: AI retires a dog this old, whatever the offer</v>
+      </c>
+      <c r="B265">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D252"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D265"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Spreadsheet row for Phase E2: every dog starts a new season fresh — snapshot unmoved
add-phase-e2-rows.ts (a copy of add-phase-e1-rows.ts) adds one row under the off-season section:
the fitness every dog starts a new season on (100), Jesse's call. Data only: nothing reads it yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017EGPNwHsuwepSCNQxqzMUS
</commit_message>
<xml_diff>
--- a/design/space_dog_racing_economy.xlsx
+++ b/design/space_dog_racing_economy.xlsx
@@ -526,7 +526,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D264"/>
+  <dimension ref="A1:D265"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2596,9 +2596,20 @@
         <v>6</v>
       </c>
     </row>
+    <row r="265">
+      <c r="A265" t="str">
+        <v>Off-season: every dog starts the new season on this fitness</v>
+      </c>
+      <c r="B265">
+        <v>100</v>
+      </c>
+      <c r="C265" t="str">
+        <v>Jesse's call for Phase E2: the off-season is a long rest. Any layoff clears too. Without it races entered fell from 2.12 a weekend in season 1 to about 1.87 after it</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D264"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D265"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add the flat stake ceiling to the sheet: 1,000 Bones a race
Phase G, Jesse's pick from the sweep. add-phase-g-rows.ts upserts the row
under Betting, balance-from-xlsx.ts maps it to `maxStake`, and balance.json
is regenerated. Nothing reads it yet, so neither golden moves.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FdrqDowiTH9hNxfsW2zev1
</commit_message>
<xml_diff>
--- a/design/space_dog_racing_economy.xlsx
+++ b/design/space_dog_racing_economy.xlsx
@@ -526,7 +526,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D265"/>
+  <dimension ref="A1:D266"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -836,379 +836,382 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Archetype finish-share assumptions (Cashflow sheet)</v>
+        <v>Max stake per race (flat ceiling, Bones)</v>
+      </c>
+      <c r="B40">
+        <v>1000</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Jesse's call for Phase G: a stable's stake on one race is the lesser of the % of cash above and this. Neon Snout doubles it. Chosen from a sweep of none / 1,000 / 1,500 / 2,000 / 3,000 / 5,000 after a two-season game was won at the bookie</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Expected share of each class's total purse a stable captures per weekend (0 = never places, 1 = wins everything).</v>
+        <v>Archetype finish-share assumptions (Cashflow sheet)</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Archetype</v>
-      </c>
-      <c r="B42" t="str">
-        <v>Bronze share</v>
-      </c>
-      <c r="C42" t="str">
-        <v>Silver share</v>
-      </c>
-      <c r="D42" t="str">
-        <v>Gold share</v>
+        <v>Expected share of each class's total purse a stable captures per weekend (0 = never places, 1 = wins everything).</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Cautious</v>
-      </c>
-      <c r="B43">
-        <v>0.3</v>
-      </c>
-      <c r="C43">
-        <v>0.15</v>
-      </c>
-      <c r="D43">
-        <v>0.05</v>
+        <v>Archetype</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Bronze share</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Silver share</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Gold share</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Average</v>
+        <v>Cautious</v>
       </c>
       <c r="B44">
-        <v>0.18</v>
+        <v>0.3</v>
       </c>
       <c r="C44">
         <v>0.15</v>
       </c>
       <c r="D44">
-        <v>0.12</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Aggressive</v>
+        <v>Average</v>
       </c>
       <c r="B45">
-        <v>0.08</v>
+        <v>0.18</v>
       </c>
       <c r="C45">
         <v>0.15</v>
       </c>
       <c r="D45">
-        <v>0.2</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
+        <v>Aggressive</v>
+      </c>
+      <c r="B46">
+        <v>0.08</v>
+      </c>
+      <c r="C46">
+        <v>0.15</v>
+      </c>
+      <c r="D46">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
         <v>Rule of thumb: a fair 8-dog field gives each stable 12.5% of the purse; a favourite ~25–35%; an outclassed dog ~3–5%.</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v>Race simulation (GDD §6.2 — the v2 rebalance, 11 September 2026)</v>
-      </c>
-      <c r="C48" t="str">
-        <v>Rebalanced so all four stats matter: measured +10-to-one-stat win rates move from speed 28.8 / stam 16.7 / accel 14.4 / trap 14.0 to rating-weight order, and track length starts to matter at all. D12.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Race: base speed (m/s)</v>
-      </c>
-      <c r="B49">
-        <v>13.75</v>
+        <v>Race simulation (GDD §6.2 — the v2 rebalance, 11 September 2026)</v>
       </c>
       <c r="C49" t="str">
-        <v>Was 13. The floor every dog runs at before its Speed stat</v>
+        <v>Rebalanced so all four stats matter: measured +10-to-one-stat win rates move from speed 28.8 / stam 16.7 / accel 14.4 / trap 14.0 to rating-weight order, and track length starts to matter at all. D12.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Race: speed coefficient (m/s per 100 Speed)</v>
+        <v>Race: base speed (m/s)</v>
       </c>
       <c r="B50">
-        <v>4.5</v>
+        <v>13.75</v>
       </c>
       <c r="C50" t="str">
-        <v>Was 6. Cutting this is what stops the race being a pure Speed contest</v>
+        <v>Was 13. The floor every dog runs at before its Speed stat</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Race: fade penalty past the stamina point</v>
+        <v>Race: speed coefficient (m/s per 100 Speed)</v>
       </c>
       <c r="B51">
-        <v>0.5</v>
+        <v>4.5</v>
       </c>
       <c r="C51" t="str">
-        <v>Was 0.35. Makes Stamina the second-biggest stat, and biggest on a stayer</v>
+        <v>Was 6. Cutting this is what stops the race being a pure Speed contest</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Race: acceleration base (m/s²)</v>
+        <v>Race: fade penalty past the stamina point</v>
       </c>
       <c r="B52">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="C52" t="str">
-        <v>Was 4. Less free acceleration, so the stat buys more</v>
+        <v>Was 0.35. Makes Stamina the second-biggest stat, and biggest on a stayer</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Race: acceleration coefficient (m/s² per 100 Accel)</v>
+        <v>Race: acceleration base (m/s²)</v>
       </c>
       <c r="B53">
-        <v>5.5</v>
+        <v>2</v>
       </c>
       <c r="C53" t="str">
-        <v>Was 6. Accel now peaks on the 350 m sprints</v>
+        <v>Was 4. Less free acceleration, so the stat buys more</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Race: break from the boxes (metres at 100 Accel)</v>
+        <v>Race: acceleration coefficient (m/s² per 100 Accel)</v>
       </c>
       <c r="B54">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="C54" t="str">
-        <v>Trap folded into Accel (GDD_V3 V9)</v>
+        <v>Was 6. Accel now peaks on the 350 m sprints</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Race: bump chance on a bend</v>
+        <v>Race: break from the boxes (metres at 100 Accel)</v>
       </c>
       <c r="B55">
-        <v>0.3</v>
+        <v>7</v>
       </c>
       <c r="C55" t="str">
-        <v>Was 0.10. The other half of what Trap buys</v>
+        <v>Trap folded into Accel (GDD_V3 V9)</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Race: bump speed penalty</v>
+        <v>Race: bump chance on a bend</v>
       </c>
       <c r="B56">
         <v>0.3</v>
       </c>
       <c r="C56" t="str">
-        <v>Was 0.15</v>
+        <v>Was 0.10. The other half of what Trap buys</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
+        <v>Race: bump speed penalty</v>
+      </c>
+      <c r="B57">
+        <v>0.3</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Was 0.15</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
         <v>Race: bump distance (metres)</v>
       </c>
-      <c r="B57">
+      <c r="B58">
         <v>1.2</v>
       </c>
-      <c r="C57" t="str">
+      <c r="C58" t="str">
         <v>Was 0.6. Dogs this close on a bend may clash</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="str">
-        <v>Condition (GDD §5.2)</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Fitness multiplier: floor</v>
-      </c>
-      <c r="B60">
-        <v>0.9</v>
-      </c>
-      <c r="C60" t="str">
-        <v>D13. Was 0.80: at equal ratings a dog at 60 fitness won 1.3% of its races, so the only usable range was 85-100 and nothing ever fell to the threshold</v>
+        <v>Condition (GDD §5.2)</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
+        <v>Fitness multiplier: floor</v>
+      </c>
+      <c r="B61">
+        <v>0.9</v>
+      </c>
+      <c r="C61" t="str">
+        <v>D13. Was 0.80: at equal ratings a dog at 60 fitness won 1.3% of its races, so the only usable range was 85-100 and nothing ever fell to the threshold</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
         <v>Fitness multiplier: range</v>
       </c>
-      <c r="B61">
+      <c r="B62">
         <v>0.1</v>
       </c>
-      <c r="C61" t="str">
+      <c r="C62" t="str">
         <v>D13. Was 0.20. Flattened, the curve reads from 40 to 100 and the weekly swings below can be big enough to see</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="str">
-        <v>Race or Rest (GDD_V3 §4.2 — the weekly per-dog state)</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Fitness: cost of a race</v>
-      </c>
-      <c r="B64">
-        <v>20</v>
-      </c>
-      <c r="C64" t="str">
-        <v>GDD_V3 §4.2 — was 25</v>
+        <v>Race or Rest (GDD_V3 §4.2 — the weekly per-dog state)</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Fitness: gain from a rest week</v>
+        <v>Fitness: cost of a race</v>
       </c>
       <c r="B65">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C65" t="str">
-        <v>GDD_V3 §4.2 — unchanged</v>
+        <v>GDD_V3 §4.2 — was 25</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Growth and decline by age (GDD_V3 §4.3)</v>
+        <v>Fitness: gain from a rest week</v>
+      </c>
+      <c r="B66">
+        <v>30</v>
+      </c>
+      <c r="C66" t="str">
+        <v>GDD_V3 §4.2 — unchanged</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Growth: stat points a week at age 1</v>
-      </c>
-      <c r="B67">
-        <v>2</v>
-      </c>
-      <c r="C67" t="str">
-        <v>Replaces v1's +1 every second week at any age up to 2. This is what makes a pup a pup</v>
+        <v>Growth and decline by age (GDD_V3 §4.3)</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Growth: stat points a week at age 2</v>
+        <v>Growth: stat points a week at age 1</v>
       </c>
       <c r="B68">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C68" t="str">
-        <v>Ages 3 and 4 neither grow nor decline</v>
+        <v>Replaces v1's +1 every second week at any age up to 2. This is what makes a pup a pup</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
+        <v>Growth: stat points a week at age 2</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Ages 3 and 4 neither grow nor decline</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
         <v>Decline: stat points a week at age 5+</v>
       </c>
-      <c r="B69">
-        <v>1</v>
-      </c>
-      <c r="C69" t="str">
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="str">
         <v>Subtracted, every week rather than every second</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="str">
-        <v>Local dogs (GDD_V3 §7.1)</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Local dog fitness</v>
-      </c>
-      <c r="B72">
-        <v>75</v>
-      </c>
-      <c r="C72" t="str">
-        <v>A planet's own runner turns up fresh but not perfect. v1 left locals on createDog's default 90, which cost nothing when campaigning stables raced at 96 and is a standing handicap now that §5.7 puts them at 60-80</v>
+        <v>Local dogs (GDD_V3 §7.1)</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Local dog rating: Gold Cup</v>
+        <v>Local dog fitness</v>
       </c>
       <c r="B73">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="C73" t="str">
-        <v>GDD_V3 §7.1 — a rich race draws a strong home team</v>
+        <v>A planet's own runner turns up fresh but not perfect. v1 left locals on createDog's default 90, which cost nothing when campaigning stables raced at 96 and is a standing handicap now that §5.7 puts them at 60-80</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Local dog rating: Silver Plate</v>
+        <v>Local dog rating: Gold Cup</v>
       </c>
       <c r="B74">
-        <v>45</v>
+        <v>55</v>
+      </c>
+      <c r="C74" t="str">
+        <v>GDD_V3 §7.1 — a rich race draws a strong home team</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
+        <v>Local dog rating: Silver Plate</v>
+      </c>
+      <c r="B75">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
         <v>Local dog rating: Bronze Dash</v>
       </c>
-      <c r="B75">
+      <c r="B76">
         <v>35</v>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="str">
+    <row r="78">
+      <c r="A78" t="str">
         <v>Information (GDD §9.3 — the fog)</v>
       </c>
-      <c r="C77" t="str">
+      <c r="C78" t="str">
         <v>The circuit is dark past next week. What you can buy back, and how far it reaches</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="str">
-        <v>The trap draw (GDD §6.2 / D37 — the rail is the short way round and where the traffic is)</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Trap draw: top-speed edge across the width of the boxes</v>
-      </c>
-      <c r="B85">
-        <v>0.018</v>
-      </c>
-      <c r="C85" t="str">
-        <v>Trap 1 runs +half of this and the outside trap −half, scaled by how tight the bends are and zero on a track with none. Symmetric, so a full field gains nothing on average — the draw redistributes a race rather than adding speed to it</v>
+        <v>The trap draw (GDD §6.2 / D37 — the rail is the short way round and where the traffic is)</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
+        <v>Trap draw: top-speed edge across the width of the boxes</v>
+      </c>
+      <c r="B86">
+        <v>0.018</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Trap 1 runs +half of this and the outside trap −half, scaled by how tight the bends are and zero on a track with none. Symmetric, so a full field gains nothing on average — the draw redistributes a race rather than adding speed to it</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
         <v>Trap draw: trap craft the rail costs, across the width of the boxes</v>
       </c>
-      <c r="B86">
+      <c r="B87">
         <v>20</v>
       </c>
-      <c r="C86" t="str">
+      <c r="C87" t="str">
         <v>A dog on the rail has less room, so it needs the craft to hold its line when two meet on a bend. Pays for the shorter trip above, and is what makes which end of the draw a dog wants depend on the dog. Replaces an accidental array-index tie-break worth 9.1% against 17.3% between identical dogs</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="str">
-        <v>The age bands (GDD_V3 §4.3 — age ticks once, in the off-season)</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Age 1: growth, stat points a week</v>
-      </c>
-      <c r="B89">
-        <v>1</v>
-      </c>
-      <c r="C89" t="str">
-        <v>Growth is ON TOP of the food (GDD_V3 §4.3)</v>
+        <v>The age bands (GDD_V3 §4.3 — age ticks once, in the off-season)</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Age 2: growth, stat points a week</v>
+        <v>Age 1: growth, stat points a week</v>
       </c>
       <c r="B90">
         <v>1</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Growth is ON TOP of the food (GDD_V3 §4.3)</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Age 5: decline, stat points a week</v>
+        <v>Age 2: growth, stat points a week</v>
       </c>
       <c r="B91">
         <v>1</v>
@@ -1216,7 +1219,7 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Age 6: decline, stat points a week</v>
+        <v>Age 5: decline, stat points a week</v>
       </c>
       <c r="B92">
         <v>1</v>
@@ -1224,7 +1227,7 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>Age 7: decline, stat points a week</v>
+        <v>Age 6: decline, stat points a week</v>
       </c>
       <c r="B93">
         <v>1</v>
@@ -1232,26 +1235,26 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Age 5: rest recovery</v>
+        <v>Age 7: decline, stat points a week</v>
       </c>
       <c r="B94">
-        <v>25</v>
-      </c>
-      <c r="C94" t="str">
-        <v>Falls from 30 — an old dog comes back slower</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>Age 6: rest recovery</v>
+        <v>Age 5: rest recovery</v>
       </c>
       <c r="B95">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Falls from 30 — an old dog comes back slower</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Age 7: rest recovery</v>
+        <v>Age 6: rest recovery</v>
       </c>
       <c r="B96">
         <v>20</v>
@@ -1259,726 +1262,726 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>Age 5: injury multiplier</v>
+        <v>Age 7: rest recovery</v>
       </c>
       <c r="B97">
-        <v>1.3</v>
-      </c>
-      <c r="C97" t="str">
-        <v>× the base 4% a race</v>
+        <v>20</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>Age 6: injury multiplier</v>
+        <v>Age 5: injury multiplier</v>
       </c>
       <c r="B98">
-        <v>1.6</v>
+        <v>1.3</v>
+      </c>
+      <c r="C98" t="str">
+        <v>× the base 4% a race</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
+        <v>Age 6: injury multiplier</v>
+      </c>
+      <c r="B99">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
         <v>Age 7: injury multiplier</v>
       </c>
-      <c r="B99">
+      <c r="B100">
         <v>2</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="str">
-        <v>The circuit (GDD_V3 §2.1 — ten weekends)</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>Major weekend</v>
-      </c>
-      <c r="B102">
-        <v>5</v>
-      </c>
-      <c r="C102" t="str">
-        <v>Purses ×2</v>
+        <v>The circuit (GDD_V3 §2.1 — ten weekends)</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>Grand Final weekend</v>
+        <v>Major weekend</v>
       </c>
       <c r="B103">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C103" t="str">
-        <v>At Collar Prime, purses ×3</v>
+        <v>Purses ×2</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>Regular planets drawn from the pool of 14</v>
+        <v>Grand Final weekend</v>
       </c>
       <c r="B104">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C104" t="str">
-        <v>⚠️ §2.1 says 9, which cannot be right — see the notes</v>
+        <v>At Collar Prime, purses ×3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
+        <v>Regular planets drawn from the pool of 14</v>
+      </c>
+      <c r="B105">
+        <v>8</v>
+      </c>
+      <c r="C105" t="str">
+        <v>⚠️ §2.1 says 9, which cannot be right — see the notes</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
         <v>Dogs dealt at the start</v>
       </c>
-      <c r="B105">
+      <c r="B106">
         <v>3</v>
       </c>
-      <c r="C105" t="str">
+      <c r="C106" t="str">
         <v>On an equal stat budget, ages 2–4 (GDD_V3 §5.5)</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="str">
-        <v>Food as the running cost (GDD_V3 §6.3, V10 — the only one there is)</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
+        <v>Food as the running cost (GDD_V3 §6.3, V10 — the only one there is)</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
         <v>Empty hold: fitness a dog loses when it does not eat</v>
       </c>
-      <c r="B108">
+      <c r="B109">
         <v>10</v>
       </c>
-      <c r="C108" t="str">
+      <c r="C109" t="str">
         <v>GDD_V3 §6.3. There is no upkeep, no wages, no fuel and no debt, so this one rule is the only thing keeping money scarce. It replaces v2’s cash penalty rather than joining it</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="str">
-        <v>The six goods (GDD_V3 §6.1 — every band is exactly 8× floor to ceiling)</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>Grey Mash: price floor</v>
-      </c>
-      <c r="B111">
-        <v>10</v>
-      </c>
-      <c r="C111" t="str">
-        <v>The ladder at the floor is 1 / 2 / 3 / 6 / 7.5 / 9</v>
+        <v>The six goods (GDD_V3 §6.1 — every band is exactly 8× floor to ceiling)</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>Grey Mash: price ceiling</v>
+        <v>Grey Mash: price floor</v>
       </c>
       <c r="B112">
-        <v>80</v>
+        <v>10</v>
+      </c>
+      <c r="C112" t="str">
+        <v>The ladder at the floor is 1 / 2 / 3 / 6 / 7.5 / 9</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>Grey Mash: shelf depth, minimum</v>
+        <v>Grey Mash: price ceiling</v>
       </c>
       <c r="B113">
-        <v>40</v>
+        <v>80</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>Grey Mash: shelf depth, maximum</v>
+        <v>Grey Mash: shelf depth, minimum</v>
       </c>
       <c r="B114">
-        <v>60</v>
+        <v>40</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>Scrapmeat: price floor</v>
+        <v>Grey Mash: shelf depth, maximum</v>
       </c>
       <c r="B115">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>Scrapmeat: price ceiling</v>
+        <v>Scrapmeat: price floor</v>
       </c>
       <c r="B116">
-        <v>160</v>
+        <v>20</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>Scrapmeat: shelf depth, minimum</v>
+        <v>Scrapmeat: price ceiling</v>
       </c>
       <c r="B117">
-        <v>30</v>
+        <v>160</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>Scrapmeat: shelf depth, maximum</v>
+        <v>Scrapmeat: shelf depth, minimum</v>
       </c>
       <c r="B118">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>Glow Tripe: price floor</v>
+        <v>Scrapmeat: shelf depth, maximum</v>
       </c>
       <c r="B119">
-        <v>30</v>
+        <v>45</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>Glow Tripe: price ceiling</v>
+        <v>Glow Tripe: price floor</v>
       </c>
       <c r="B120">
-        <v>240</v>
+        <v>30</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>Glow Tripe: shelf depth, minimum</v>
+        <v>Glow Tripe: price ceiling</v>
       </c>
       <c r="B121">
-        <v>20</v>
+        <v>240</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>Glow Tripe: shelf depth, maximum</v>
+        <v>Glow Tripe: shelf depth, minimum</v>
       </c>
       <c r="B122">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>Vat Steak: price floor</v>
+        <v>Glow Tripe: shelf depth, maximum</v>
       </c>
       <c r="B123">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>Vat Steak: price ceiling</v>
+        <v>Vat Steak: price floor</v>
       </c>
       <c r="B124">
-        <v>480</v>
+        <v>60</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>Vat Steak: shelf depth, minimum</v>
+        <v>Vat Steak: price ceiling</v>
       </c>
       <c r="B125">
-        <v>10</v>
+        <v>480</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>Vat Steak: shelf depth, maximum</v>
+        <v>Vat Steak: shelf depth, minimum</v>
       </c>
       <c r="B126">
-        <v>18</v>
+        <v>10</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>Pulsar Marrow: price floor</v>
+        <v>Vat Steak: shelf depth, maximum</v>
       </c>
       <c r="B127">
-        <v>75</v>
+        <v>18</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>Pulsar Marrow: price ceiling</v>
+        <v>Pulsar Marrow: price floor</v>
       </c>
       <c r="B128">
-        <v>600</v>
+        <v>75</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>Pulsar Marrow: shelf depth, minimum</v>
+        <v>Pulsar Marrow: price ceiling</v>
       </c>
       <c r="B129">
-        <v>6</v>
+        <v>600</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>Pulsar Marrow: shelf depth, maximum</v>
+        <v>Pulsar Marrow: shelf depth, minimum</v>
       </c>
       <c r="B130">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>Ambrosia: price floor</v>
+        <v>Pulsar Marrow: shelf depth, maximum</v>
       </c>
       <c r="B131">
-        <v>90</v>
+        <v>12</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>Ambrosia: price ceiling</v>
+        <v>Ambrosia: price floor</v>
       </c>
       <c r="B132">
-        <v>720</v>
+        <v>90</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>Ambrosia: shelf depth, minimum</v>
+        <v>Ambrosia: price ceiling</v>
       </c>
       <c r="B133">
-        <v>3</v>
+        <v>720</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
+        <v>Ambrosia: shelf depth, minimum</v>
+      </c>
+      <c r="B134">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
         <v>Ambrosia: shelf depth, maximum</v>
       </c>
-      <c r="B134">
+      <c r="B135">
         <v>8</v>
       </c>
-      <c r="C134" t="str">
+      <c r="C135" t="str">
         <v>V7: the scarcity rule. ~8 units a planet, so the big trade has to be assembled over several weeks under a fog</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="str">
-        <v>Food as training (GDD_V3 §6.3 — what one week of each food does)</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>Grey Mash: stat points a week, minimum</v>
-      </c>
-      <c r="B137">
-        <v>1</v>
+        <v>Food as training (GDD_V3 §6.3 — what one week of each food does)</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>Grey Mash: stat points a week, maximum</v>
+        <v>Grey Mash: stat points a week, minimum</v>
       </c>
       <c r="B138">
         <v>1</v>
-      </c>
-      <c r="C138" t="str">
-        <v>Lands on a random stat — the floor of improvement a stable that spends nothing still gets</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>Scrapmeat: stat points a week, minimum</v>
+        <v>Grey Mash: stat points a week, maximum</v>
       </c>
       <c r="B139">
         <v>1</v>
+      </c>
+      <c r="C139" t="str">
+        <v>Lands on a random stat — the floor of improvement a stable that spends nothing still gets</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>Scrapmeat: stat points a week, maximum</v>
+        <v>Scrapmeat: stat points a week, minimum</v>
       </c>
       <c r="B140">
-        <v>2</v>
-      </c>
-      <c r="C140" t="str">
-        <v>Stamina</v>
+        <v>1</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>Glow Tripe: stat points a week, minimum</v>
+        <v>Scrapmeat: stat points a week, maximum</v>
       </c>
       <c r="B141">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="C141" t="str">
+        <v>Stamina</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>Glow Tripe: stat points a week, maximum</v>
+        <v>Glow Tripe: stat points a week, minimum</v>
       </c>
       <c r="B142">
-        <v>3</v>
-      </c>
-      <c r="C142" t="str">
-        <v>Acceleration</v>
+        <v>1</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>Vat Steak: stat points a week, minimum</v>
+        <v>Glow Tripe: stat points a week, maximum</v>
       </c>
       <c r="B143">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="C143" t="str">
+        <v>Acceleration</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>Vat Steak: stat points a week, maximum</v>
+        <v>Vat Steak: stat points a week, minimum</v>
       </c>
       <c r="B144">
-        <v>4</v>
-      </c>
-      <c r="C144" t="str">
-        <v>Speed</v>
+        <v>2</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>Pulsar Marrow: stat points a week, minimum</v>
+        <v>Vat Steak: stat points a week, maximum</v>
       </c>
       <c r="B145">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="C145" t="str">
+        <v>Speed</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>Pulsar Marrow: stat points a week, maximum</v>
+        <v>Pulsar Marrow: stat points a week, minimum</v>
       </c>
       <c r="B146">
-        <v>4</v>
-      </c>
-      <c r="C146" t="str">
-        <v>Random stat, and it touches condition</v>
+        <v>2</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>Pulsar Marrow: fitness a week</v>
+        <v>Pulsar Marrow: stat points a week, maximum</v>
       </c>
       <c r="B147">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="C147" t="str">
+        <v>Random stat, and it touches condition</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>Ambrosia: stat points a week, minimum</v>
+        <v>Pulsar Marrow: fitness a week</v>
       </c>
       <c r="B148">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>Ambrosia: stat points a week, maximum</v>
+        <v>Ambrosia: stat points a week, minimum</v>
       </c>
       <c r="B149">
-        <v>6</v>
-      </c>
-      <c r="C149" t="str">
-        <v>Random stat, condition, and injury chance halved this week</v>
+        <v>3</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>Ambrosia: fitness a week</v>
+        <v>Ambrosia: stat points a week, maximum</v>
       </c>
       <c r="B150">
-        <v>8</v>
+        <v>6</v>
+      </c>
+      <c r="C150" t="str">
+        <v>Random stat, condition, and injury chance halved this week</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
+        <v>Ambrosia: fitness a week</v>
+      </c>
+      <c r="B151">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
         <v>Ambrosia: injury chance multiplier for the week</v>
       </c>
-      <c r="B151">
+      <c r="B152">
         <v>0.5</v>
       </c>
-      <c r="C151" t="str">
+      <c r="C152" t="str">
         <v>GDD_V3 §6.3 — halved</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="str">
-        <v>The price distribution (GDD_V3 §6.4 — the row that protects the game)</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>Price draw: standard deviation as a fraction of the band</v>
-      </c>
-      <c r="B154">
-        <v>0.16</v>
-      </c>
-      <c r="C154" t="str">
-        <v>GDD_V3 §6.4: prices cluster mid-band with RARE excursions to the ends, so the 8× is something a player hunts rather than something that happens to them. At 0.16, on a planet that prices the good mid-band, a draw reaches the outer twentieth of the band about one time in four hundred at either end</v>
+        <v>The price distribution (GDD_V3 §6.4 — the row that protects the game)</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>Price draw: clamp, closest a draw may come to either end of the band</v>
+        <v>Price draw: standard deviation as a fraction of the band</v>
       </c>
       <c r="B155">
-        <v>0.02</v>
+        <v>0.16</v>
       </c>
       <c r="C155" t="str">
-        <v>As a fraction of the band. A normal deviate is unbounded; the band is not, and §6.1’s 8× is a hard global range</v>
+        <v>GDD_V3 §6.4: prices cluster mid-band with RARE excursions to the ends, so the 8× is something a player hunts rather than something that happens to them. At 0.16, on a planet that prices the good mid-band, a draw reaches the outer twentieth of the band about one time in four hundred at either end</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>Planet band bias: floor</v>
+        <v>Price draw: clamp, closest a draw may come to either end of the band</v>
       </c>
       <c r="B156">
-        <v>0.45</v>
+        <v>0.02</v>
       </c>
       <c r="C156" t="str">
-        <v>A planet’s per-good multiplier over the mid-band centre (GDD_V3 §12). Clamped to this range so every planet can still throw an excursion to either end</v>
+        <v>As a fraction of the band. A normal deviate is unbounded; the band is not, and §6.1’s 8× is a hard global range</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
+        <v>Planet band bias: floor</v>
+      </c>
+      <c r="B157">
+        <v>0.45</v>
+      </c>
+      <c r="C157" t="str">
+        <v>A planet’s per-good multiplier over the mid-band centre (GDD_V3 §12). Clamped to this range so every planet can still throw an excursion to either end</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
         <v>Planet band bias: ceiling</v>
       </c>
-      <c r="B157">
+      <c r="B158">
         <v>1.55</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="str">
-        <v>Running styles (GDD_V3 §5.1–5.2 — a redistribution of the same energy, not a bonus)</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>Front-runner: early top-speed multiplier</v>
-      </c>
-      <c r="B160">
-        <v>1.08</v>
-      </c>
-      <c r="C160" t="str">
-        <v>Bursts from the boxes, leads early, pays for it later. Leans on Acceleration</v>
+        <v>Running styles (GDD_V3 §5.1–5.2 — a redistribution of the same energy, not a bonus)</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>Front-runner: fade start shift</v>
+        <v>Front-runner: early top-speed multiplier</v>
       </c>
       <c r="B161">
-        <v>-0.05</v>
+        <v>1.08</v>
       </c>
       <c r="C161" t="str">
-        <v>In the same units as the fade point itself; negative is earlier. −0.07 at v3c; eased at v3c2 (C13) because the hot pace now burns front-runners that go together</v>
+        <v>Bursts from the boxes, leads early, pays for it later. Leans on Acceleration</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>Front-runner: fade penalty multiplier</v>
+        <v>Front-runner: fade start shift</v>
       </c>
       <c r="B162">
-        <v>1</v>
+        <v>-0.05</v>
+      </c>
+      <c r="C162" t="str">
+        <v>In the same units as the fade point itself; negative is earlier. −0.07 at v3c; eased at v3c2 (C13) because the hot pace now burns front-runners that go together</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>Stalker: early top-speed multiplier</v>
+        <v>Front-runner: fade penalty multiplier</v>
       </c>
       <c r="B163">
         <v>1</v>
-      </c>
-      <c r="C163" t="str">
-        <v>The baseline: even pace, sits handy, wins by being better. Leans on Speed</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>Stalker: fade start shift</v>
+        <v>Stalker: early top-speed multiplier</v>
       </c>
       <c r="B164">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="C164" t="str">
+        <v>The baseline: even pace, sits handy, wins by being better. Leans on Speed</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>Stalker: fade penalty multiplier</v>
+        <v>Stalker: fade start shift</v>
       </c>
       <c r="B165">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>Closer: early top-speed multiplier</v>
+        <v>Stalker: fade penalty multiplier</v>
       </c>
       <c r="B166">
-        <v>0.97</v>
-      </c>
-      <c r="C166" t="str">
-        <v>Slow away, comes home hardest. Leans on Stamina</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>Closer: fade start shift</v>
+        <v>Closer: early top-speed multiplier</v>
       </c>
       <c r="B167">
-        <v>0.035</v>
+        <v>0.97</v>
       </c>
       <c r="C167" t="str">
-        <v>+0.06 at v3c; trimmed at v3c2 to +0.04 (C13) because the hot pace now hands the closer the wins crowded front-runners lose, and to +0.035 (C14) because the run-in favours whoever is quickest over the last metres</v>
+        <v>Slow away, comes home hardest. Leans on Stamina</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>Closer: fade penalty multiplier</v>
+        <v>Closer: fade start shift</v>
       </c>
       <c r="B168">
-        <v>1</v>
+        <v>0.035</v>
+      </c>
+      <c r="C168" t="str">
+        <v>+0.06 at v3c; trimmed at v3c2 to +0.04 (C13) because the hot pace now hands the closer the wins crowded front-runners lose, and to +0.035 (C14) because the run-in favours whoever is quickest over the last metres</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>Style: the early part of the race (fraction of the trip)</v>
+        <v>Closer: fade penalty multiplier</v>
       </c>
       <c r="B169">
-        <v>0.333</v>
-      </c>
-      <c r="C169" t="str">
-        <v>Where the early top-speed multiplier applies. The first third of the trip</v>
+        <v>1</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>Style expression: minimum</v>
+        <v>Style: the early part of the race (fraction of the trip)</v>
       </c>
       <c r="B170">
-        <v>0.3</v>
+        <v>0.333</v>
       </c>
       <c r="C170" t="str">
-        <v>GDD_V3 §5.2, V13: one U(min, max) draw per runner per race, scaling how strongly its style applies that day. NOT a multiplier on speed — the area under the curve stays put and only its shape moves</v>
+        <v>Where the early top-speed multiplier applies. The first third of the trip</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
+        <v>Style expression: minimum</v>
+      </c>
+      <c r="B171">
+        <v>0.3</v>
+      </c>
+      <c r="C171" t="str">
+        <v>GDD_V3 §5.2, V13: one U(min, max) draw per runner per race, scaling how strongly its style applies that day. NOT a multiplier on speed — the area under the curve stays put and only its shape moves</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="str">
         <v>Style expression: maximum</v>
       </c>
-      <c r="B171">
+      <c r="B172">
         <v>1.3</v>
       </c>
     </row>
-    <row r="173">
-      <c r="A173" t="str">
+    <row r="174">
+      <c r="A174" t="str">
         <v>The contest rule (GDD_V3 §5.3 — a kill switch, not a tuning target)</v>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="str">
-        <v>The opening hand (GDD_V3 §5.5 — equal strength, different shapes)</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>Starting dog rating (every dealt dog, exactly)</v>
-      </c>
-      <c r="B176">
-        <v>50</v>
-      </c>
-      <c r="C176" t="str">
-        <v>V2’s promise, kept by the rating rather than by a stat total: with weights of 0.40 / 0.35 / 0.25, an equal total dealt dogs rated 44–55 (Phase B, correction 3)</v>
+        <v>The opening hand (GDD_V3 §5.5 — equal strength, different shapes)</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
+        <v>Starting dog rating (every dealt dog, exactly)</v>
+      </c>
+      <c r="B177">
+        <v>50</v>
+      </c>
+      <c r="C177" t="str">
+        <v>V2’s promise, kept by the rating rather than by a stat total: with weights of 0.40 / 0.35 / 0.25, an equal total dealt dogs rated 44–55 (Phase B, correction 3)</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
         <v>Starting dog shape: widest deviation on speed or accel</v>
       </c>
-      <c r="B177">
+      <c r="B178">
         <v>15</v>
       </c>
-      <c r="C177" t="str">
+      <c r="C178" t="str">
         <v>Speed and accel are each drawn within this of the rating, and stamina solves for it — so a dealt dog can be a speed dog, an accel dog or a stamina dog, and never a better one</v>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="str">
-        <v>The fade in metres (A7, GDD_V3 B9 — stamina has to be worth more on a staying trip)</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>Race: reference trip for the fade point (metres)</v>
-      </c>
-      <c r="B180">
-        <v>600</v>
-      </c>
-      <c r="C180" t="str">
-        <v>The fade point was a fraction of the trip (0.45 + 0.45 × stamina/100). It is now that fraction of THIS many metres, whatever the trip — so a staying trip runs past it and a sprint barely reaches it</v>
+        <v>The fade in metres (A7, GDD_V3 B9 — stamina has to be worth more on a staying trip)</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
+        <v>Race: reference trip for the fade point (metres)</v>
+      </c>
+      <c r="B181">
+        <v>600</v>
+      </c>
+      <c r="C181" t="str">
+        <v>The fade point was a fraction of the trip (0.45 + 0.45 × stamina/100). It is now that fraction of THIS many metres, whatever the trip — so a staying trip runs past it and a sprint barely reaches it</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
         <v>Race: metres from the fade point to a full fade</v>
       </c>
-      <c r="B181">
+      <c r="B182">
         <v>250</v>
       </c>
-      <c r="C181" t="str">
+      <c r="C182" t="str">
         <v>The rate a tiring dog slows at: the fade penalty is reached this far past the fade point, and held from there to the line</v>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="str">
-        <v>The bookie and running styles (GDD_V3 §5.6 — the style and the trip, never the field)</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>Book: Front-runner on a sprint (rating points)</v>
-      </c>
-      <c r="B184">
-        <v>4</v>
-      </c>
-      <c r="C184" t="str">
-        <v>Fitted by --styles at oddsScale 18.75: 18.1% of eight-dog sprints and 6.5% of staying trips, against 12.5% even</v>
+        <v>The bookie and running styles (GDD_V3 §5.6 — the style and the trip, never the field)</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>Book: Front-runner on a standard trip (rating points)</v>
+        <v>Book: Front-runner on a sprint (rating points)</v>
       </c>
       <c r="B185">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="C185" t="str">
+        <v>Fitted by --styles at oddsScale 18.75: 18.1% of eight-dog sprints and 6.5% of staying trips, against 12.5% even</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>Book: Front-runner on a staying trip (rating points)</v>
+        <v>Book: Front-runner on a standard trip (rating points)</v>
       </c>
       <c r="B186">
-        <v>-6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>Book: Stalker on a sprint (rating points)</v>
+        <v>Book: Front-runner on a staying trip (rating points)</v>
       </c>
       <c r="B187">
-        <v>-1</v>
-      </c>
-      <c r="C187" t="str">
-        <v>Fitted: 11.0% sprint, 11.9% staying</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>Book: Stalker on a standard trip (rating points)</v>
+        <v>Book: Stalker on a sprint (rating points)</v>
       </c>
       <c r="B188">
-        <v>0</v>
+        <v>-1</v>
+      </c>
+      <c r="C188" t="str">
+        <v>Fitted: 11.0% sprint, 11.9% staying</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>Book: Stalker on a staying trip (rating points)</v>
+        <v>Book: Stalker on a standard trip (rating points)</v>
       </c>
       <c r="B189">
         <v>0</v>
@@ -1986,334 +1989,334 @@
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>Book: Closer on a sprint (rating points)</v>
+        <v>Book: Stalker on a staying trip (rating points)</v>
       </c>
       <c r="B190">
-        <v>-4</v>
-      </c>
-      <c r="C190" t="str">
-        <v>Fitted: 8.4% sprint, 19.1% staying</v>
+        <v>0</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>Book: Closer on a standard trip (rating points)</v>
+        <v>Book: Closer on a sprint (rating points)</v>
       </c>
       <c r="B191">
-        <v>0</v>
+        <v>-4</v>
+      </c>
+      <c r="C191" t="str">
+        <v>Fitted: 8.4% sprint, 19.1% staying</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
+        <v>Book: Closer on a standard trip (rating points)</v>
+      </c>
+      <c r="B192">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
         <v>Book: Closer on a staying trip (rating points)</v>
       </c>
-      <c r="B192">
+      <c r="B193">
         <v>4</v>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="str">
-        <v>The hot pace (GDD_V3 §5.3 — two front-runners at the head light it; the lead group pays)</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>Hot pace: window (fraction of the trip)</v>
-      </c>
-      <c r="B195">
-        <v>0.333</v>
-      </c>
-      <c r="C195" t="str">
-        <v>The pace can only be hot while the leader is inside this much of the trip. The first third, as for the style curve</v>
+        <v>The hot pace (GDD_V3 §5.3 — two front-runners at the head light it; the lead group pays)</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v>Hot pace: front-runners within this of each other at the head (metres)</v>
+        <v>Hot pace: window (fraction of the trip)</v>
       </c>
       <c r="B196">
-        <v>4</v>
+        <v>0.333</v>
       </c>
       <c r="C196" t="str">
-        <v>Two or more runners whose style lights the pace, both this close to the leader (so to each other), make the pace hot. One alone never does</v>
+        <v>The pace can only be hot while the leader is inside this much of the trip. The first third, as for the style curve</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v>Hot pace: the lead group, within this of the leader (metres)</v>
+        <v>Hot pace: front-runners within this of each other at the head (metres)</v>
       </c>
       <c r="B197">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C197" t="str">
-        <v>While the pace is hot, every runner this close to the leader pays — front-runners and the stalkers sitting on them alike. A dog further back pays nothing</v>
+        <v>Two or more runners whose style lights the pace, both this close to the leader (so to each other), make the pace hot. One alone never does</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>Hot pace: fade point cost for a whole window in a hot lead group (metres)</v>
+        <v>Hot pace: the lead group, within this of the leader (metres)</v>
       </c>
       <c r="B198">
-        <v>90</v>
+        <v>6</v>
       </c>
       <c r="C198" t="str">
-        <v>Pro rata to the ground a dog covers in the lead group while the pace is hot. Metres, like the fade point itself (A7)</v>
+        <v>While the pace is hot, every runner this close to the leader pays — front-runners and the stalkers sitting on them alike. A dog further back pays nothing</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>Front-runner: lights the pace (1 = yes)</v>
+        <v>Hot pace: fade point cost for a whole window in a hot lead group (metres)</v>
       </c>
       <c r="B199">
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="C199" t="str">
-        <v>A style is a row: the rule counts runners whose style says 1 here, and never asks a style its name</v>
+        <v>Pro rata to the ground a dog covers in the lead group while the pace is hot. Metres, like the fade point itself (A7)</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v>Stalker: lights the pace (1 = yes)</v>
+        <v>Front-runner: lights the pace (1 = yes)</v>
       </c>
       <c r="B200">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="C200" t="str">
+        <v>A style is a row: the rule counts runners whose style says 1 here, and never asks a style its name</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>Closer: lights the pace (1 = yes)</v>
+        <v>Stalker: lights the pace (1 = yes)</v>
       </c>
       <c r="B201">
         <v>0</v>
       </c>
     </row>
-    <row r="203">
-      <c r="A203" t="str">
-        <v>The run-in (GDD_V3 §7.2, §14 Q11 — the whole field tires into the line; nobody is pulled back)</v>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>Closer: lights the pace (1 = yes)</v>
+      </c>
+      <c r="B202">
+        <v>0</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>Race: the run-in, the last metres of every trip (metres)</v>
-      </c>
-      <c r="B204">
-        <v>15</v>
-      </c>
-      <c r="C204" t="str">
-        <v>Over these last metres every runner slows by the same fraction at the same point on the track, reaching the loss below at the line. Keyed to where a dog is, never to where the others are</v>
+        <v>The run-in (GDD_V3 §7.2, §14 Q11 — the whole field tires into the line; nobody is pulled back)</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
+        <v>Race: the run-in, the last metres of every trip (metres)</v>
+      </c>
+      <c r="B205">
+        <v>15</v>
+      </c>
+      <c r="C205" t="str">
+        <v>Over these last metres every runner slows by the same fraction at the same point on the track, reaching the loss below at the line. Keyed to where a dog is, never to where the others are</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
         <v>Race: speed lost at the line in the run-in</v>
       </c>
-      <c r="B205">
+      <c r="B206">
         <v>0.5</v>
       </c>
-      <c r="C205" t="str">
+      <c r="C206" t="str">
         <v>What the fade in fractions (v3b) did to the whole field before A7 made the fade metres: a time gap stays a time gap, and the metres it shows at the line shrink with the speed</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="str">
-        <v>Dog offers (GDD_V3 §9.2 — age, one stat, and patter that is sometimes a lie)</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
-        <v>Dog offer: the seller lies, chance</v>
-      </c>
-      <c r="B208">
-        <v>0.35</v>
-      </c>
-      <c r="C208" t="str">
-        <v>Before the card row's own multiplier: a monk never lies (×0), a man in a long coat usually does. A lie is a claimed stat that is really poor</v>
+        <v>Dog offers (GDD_V3 §9.2 — age, one stat, and patter that is sometimes a lie)</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
-        <v>Dog offer: rating, mean</v>
+        <v>Dog offer: the seller lies, chance</v>
       </c>
       <c r="B209">
-        <v>42</v>
+        <v>0.35</v>
       </c>
       <c r="C209" t="str">
-        <v>Where an offered dog's stats centre. A dealt dog rates 50, so the average offer is a step down and the gamble is the spread and the patter. 50 at first; 44 in Phase D1, and then 42, because at 50 the Pound alone lifted mean end worth about 2,000 and out of its 25-40k band, and at 44 it sat on the 40k line</v>
+        <v>Before the card row's own multiplier: a monk never lies (×0), a man in a long coat usually does. A lie is a claimed stat that is really poor</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
-        <v>Dog offer: rating, sd</v>
+        <v>Dog offer: rating, mean</v>
       </c>
       <c r="B210">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="C210" t="str">
-        <v>Spread of the offered dog's level, before its shape. Rating is never shown</v>
+        <v>Where an offered dog's stats centre. A dealt dog rates 50, so the average offer is a step down and the gamble is the spread and the patter. 50 at first; 44 in Phase D1, and then 42, because at 50 the Pound alone lifted mean end worth about 2,000 and out of its 25-40k band, and at 44 it sat on the 40k line</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v>Dog offer: youngest age</v>
+        <v>Dog offer: rating, sd</v>
       </c>
       <c r="B211">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="C211" t="str">
+        <v>Spread of the offered dog's level, before its shape. Rating is never shown</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v>Dog offer: oldest age</v>
+        <v>Dog offer: youngest age</v>
       </c>
       <c r="B212">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v>Dog offer: the claimed stat, when honest (points above the level)</v>
+        <v>Dog offer: oldest age</v>
       </c>
       <c r="B213">
-        <v>10</v>
-      </c>
-      <c r="C213" t="str">
-        <v>The seller talks up one stat you cannot see. Honest, it really is this far above the dog's level</v>
+        <v>6</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
+        <v>Dog offer: the claimed stat, when honest (points above the level)</v>
+      </c>
+      <c r="B214">
+        <v>10</v>
+      </c>
+      <c r="C214" t="str">
+        <v>The seller talks up one stat you cannot see. Honest, it really is this far above the dog's level</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
         <v>Dog offer: the claimed stat, when lying (points below the level)</v>
       </c>
-      <c r="B214">
+      <c r="B215">
         <v>12</v>
       </c>
-      <c r="C214" t="str">
+      <c r="C215" t="str">
         <v>Lying, the stat he talks up is this far below it</v>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="str">
-        <v>Race-day conditions (Phase D1 — drawn on arrival, applied on race day, never priced by the book)</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
-        <v>Condition: a knock, chance per stable dog per weekend</v>
-      </c>
-      <c r="B217">
-        <v>0.06</v>
-      </c>
-      <c r="C217" t="str">
-        <v>Drawn for every stable dog at arrival, one draw a dog whatever it lands on, so the stream never depends on the outcome</v>
+        <v>Race-day conditions (Phase D1 — drawn on arrival, applied on race day, never priced by the book)</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
-        <v>Condition: a knock, fitness on race day</v>
+        <v>Condition: a knock, chance per stable dog per weekend</v>
       </c>
       <c r="B218">
-        <v>-30</v>
+        <v>0.06</v>
       </c>
       <c r="C218" t="str">
-        <v>Applied to the runner, never to the stored fitness: every screen and the whole book go on reading the dog as it was</v>
+        <v>Drawn for every stable dog at arrival, one draw a dog whatever it lands on, so the stream never depends on the outcome</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
-        <v>Condition: off its feed, chance per stable dog per weekend</v>
+        <v>Condition: a knock, fitness on race day</v>
       </c>
       <c r="B219">
-        <v>0.06</v>
+        <v>-30</v>
+      </c>
+      <c r="C219" t="str">
+        <v>Applied to the runner, never to the stored fitness: every screen and the whole book go on reading the dog as it was</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
-        <v>Condition: off its feed, fitness on race day</v>
+        <v>Condition: off its feed, chance per stable dog per weekend</v>
       </c>
       <c r="B220">
-        <v>-15</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
-        <v>Condition: buzzing, chance per stable dog per weekend</v>
+        <v>Condition: off its feed, fitness on race day</v>
       </c>
       <c r="B221">
-        <v>0.08</v>
+        <v>-15</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
+        <v>Condition: buzzing, chance per stable dog per weekend</v>
+      </c>
+      <c r="B222">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="str">
         <v>Condition: buzzing, speed on race day (stat points)</v>
       </c>
-      <c r="B222">
+      <c r="B223">
         <v>3</v>
       </c>
-      <c r="C222" t="str">
+      <c r="C223" t="str">
         <v>Like the lucky bone, but nobody knows unless tipped — the owner included. 8 read +53% a Bone backed, 5 read +33% and 4 +32% at 800 seasons (the standard error is about 4 points); 3 is the setting</v>
       </c>
     </row>
-    <row r="224">
-      <c r="A224" t="str">
+    <row r="225">
+      <c r="A225" t="str">
         <v>The free local runner (GDD_V3 §4.4 — a stable short of fit dogs is lent one)</v>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="str">
-        <v>Staff (GDD_V3 §8 — two trainers, paid a cut of race prize money only)</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
-        <v>Staff: trainers dealt to each stable at the start of a game</v>
-      </c>
-      <c r="B227">
-        <v>2</v>
-      </c>
-      <c r="C227" t="str">
-        <v>Two slots, everyone a trainer (§8.1). Dealt at createSeason from the staff rows; the only way to change one in Phase D is a Bar card</v>
+        <v>Staff (GDD_V3 §8 — two trainers, paid a cut of race prize money only)</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
-        <v>Staff cut: +1 stat a week</v>
+        <v>Staff: trainers dealt to each stable at the start of a game</v>
       </c>
       <c r="B228">
-        <v>0.03</v>
+        <v>2</v>
       </c>
       <c r="C228" t="str">
-        <v>Commission, a share of race prize money only (§8.1). A trainer with one bonus takes its cut; with two, the sum plus the premium below, capped</v>
+        <v>Two slots, everyone a trainer (§8.1). Dealt at createSeason from the staff rows; the only way to change one in Phase D is a Bar card</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
-        <v>Staff cut: +5 fitness recovery a week</v>
+        <v>Staff cut: +1 stat a week</v>
       </c>
       <c r="B229">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="C229" t="str">
-        <v>3% at first. Measured at 800 seasons by regressing end worth on the dealt bonuses (the deal is random, so it is a clean experiment): a +5-recovery trainer was worth ~1,300 to its stable at 3%. 5% leaves it worth having</v>
+        <v>Commission, a share of race prize money only (§8.1). A trainer with one bonus takes its cut; with two, the sum plus the premium below, capped</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
-        <v>Staff cut: injury chance halved</v>
+        <v>Staff cut: +5 fitness recovery a week</v>
       </c>
       <c r="B230">
-        <v>0.04</v>
+        <v>0.05</v>
+      </c>
+      <c r="C230" t="str">
+        <v>3% at first. Measured at 800 seasons by regressing end worth on the dealt bonuses (the deal is random, so it is a clean experiment): a +5-recovery trainer was worth ~1,300 to its stable at 3%. 5% leaves it worth having</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
-        <v>Staff cut: injury duration −1 week</v>
+        <v>Staff cut: injury chance halved</v>
       </c>
       <c r="B231">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
-        <v>Staff cut: reveals a rival dog's style a week</v>
+        <v>Staff cut: injury duration −1 week</v>
       </c>
       <c r="B232">
         <v>0.02</v>
@@ -2321,295 +2324,303 @@
     </row>
     <row r="233">
       <c r="A233" t="str">
-        <v>Staff cut: next planet's band position for all six goods</v>
+        <v>Staff cut: reveals a rival dog's style a week</v>
       </c>
       <c r="B233">
-        <v>0.08</v>
-      </c>
-      <c r="C233" t="str">
-        <v>3% at first, and it was the cheapest bonus in the pool for what it did: knowing all six of next week's prices every week lifted food's share of gross income four points and was worth ~1,000 to its stable. At 8% the regression reads it at nothing either way — the same 8% trainer is cheap for a trader and dear for a racer (§8.1)</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
-        <v>Staff cut: +10% prize money</v>
+        <v>Staff cut: next planet's band position for all six goods</v>
       </c>
       <c r="B234">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="C234" t="str">
-        <v>5% at first; 6% after the 800-season regression</v>
+        <v>3% at first, and it was the cheapest bonus in the pool for what it did: knowing all six of next week's prices every week lifted food's share of gross income four points and was worth ~1,000 to its stable. At 8% the regression reads it at nothing either way — the same 8% trainer is cheap for a trader and dear for a racer (§8.1)</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
-        <v>Staff cut: Explore less likely to go badly</v>
+        <v>Staff cut: +10% prize money</v>
       </c>
       <c r="B235">
-        <v>0.03</v>
+        <v>0.06</v>
+      </c>
+      <c r="C235" t="str">
+        <v>5% at first; 6% after the 800-season regression</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
-        <v>Staff cut: premium for a trainer with two bonuses</v>
+        <v>Staff cut: Explore less likely to go badly</v>
       </c>
       <c r="B236">
-        <v>0.02</v>
-      </c>
-      <c r="C236" t="str">
-        <v>§8.2: "two of the above, 6–10%". The cheapest pair (2% + 2%) lands on 6%</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
-        <v>Staff cut: the most a trainer takes</v>
+        <v>Staff cut: premium for a trainer with two bonuses</v>
       </c>
       <c r="B237">
-        <v>0.1</v>
+        <v>0.02</v>
       </c>
       <c r="C237" t="str">
-        <v>§8.1: 1–10%. A 10% trainer on a stable earning 30,000 in purses costs 3,000</v>
+        <v>§8.2: "two of the above, 6–10%". The cheapest pair (2% + 2%) lands on 6%</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
-        <v>Staff bonus: fitness a week, to a dog that did not run</v>
+        <v>Staff cut: the most a trainer takes</v>
       </c>
       <c r="B238">
-        <v>5</v>
+        <v>0.1</v>
       </c>
       <c r="C238" t="str">
-        <v>Folded into weeklyFitnessDelta's bonus, so it goes through the week's one clamp</v>
+        <v>§8.1: 1–10%. A 10% trainer on a stable earning 30,000 in purses costs 3,000</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
-        <v>Staff bonus: injury chance ×</v>
+        <v>Staff bonus: fitness a week, to a dog that did not run</v>
       </c>
       <c r="B239">
-        <v>0.5</v>
+        <v>5</v>
+      </c>
+      <c r="C239" t="str">
+        <v>Folded into weeklyFitnessDelta's bonus, so it goes through the week's one clamp</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
-        <v>Staff bonus: weeks off a layoff, at the roll</v>
+        <v>Staff bonus: injury chance ×</v>
       </c>
       <c r="B240">
-        <v>1</v>
-      </c>
-      <c r="C240" t="str">
-        <v>Never below one week</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
-        <v>Staff bonus: extra prize money, share of the purse</v>
+        <v>Staff bonus: weeks off a layoff, at the roll</v>
       </c>
       <c r="B241">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="C241" t="str">
-        <v>Added before the commission is taken</v>
+        <v>Never below one week</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
-        <v>Staff bonus: an Explore card's bad-outcome chance ×</v>
+        <v>Staff bonus: extra prize money, share of the purse</v>
       </c>
       <c r="B242">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="C242" t="str">
-        <v>Read by every card through the kit's risk() and luck() helpers, never by a branch</v>
+        <v>Added before the commission is taken</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
+        <v>Staff bonus: an Explore card's bad-outcome chance ×</v>
+      </c>
+      <c r="B243">
+        <v>0.5</v>
+      </c>
+      <c r="C243" t="str">
+        <v>Read by every card through the kit's risk() and luck() helpers, never by a branch</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
         <v>Staff bonus: stat points a week, to one dog</v>
       </c>
-      <c r="B243">
-        <v>1</v>
-      </c>
-      <c r="C243" t="str">
+      <c r="B244">
+        <v>1</v>
+      </c>
+      <c r="C244" t="str">
         <v>§8.2's "+1 to one stat per week": at the jump, beside the food, on the lowest-rated dog's weakest stat by the rating's weights — a rule, not a draw. Built first as +1 to every dog, which made a 3% trainer worth ~4,000 of end worth and took mean end worth out of its band (decision D10)</v>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" t="str">
-        <v>Sabotage (GDD_V3 §9.3 — a nobble, a bought box, and the stewards who might notice)</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>Sabotage: a nobbled runner's fitness on race day</v>
-      </c>
-      <c r="B246">
-        <v>-25</v>
-      </c>
-      <c r="C246" t="str">
-        <v>Applied to the runner, like a race-day condition: the book has struck its prices and the victim's stated fitness never changes</v>
+        <v>Sabotage (GDD_V3 §9.3 — a nobble, a bought box, and the stewards who might notice)</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>Sabotage: stewards catch a nobbler, chance (any planet without its own)</v>
+        <v>Sabotage: a nobbled runner's fitness on race day</v>
       </c>
       <c r="B247">
-        <v>0.35</v>
+        <v>-25</v>
       </c>
       <c r="C247" t="str">
-        <v>Rolled on race day from one draw per stable, made every week whether or not anybody booked a job, so the game stream never depends on a door</v>
+        <v>Applied to the runner, like a race-day condition: the book has struck its prices and the victim's stated fitness never changes</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>Sabotage: catch chance at Lagrange Lows</v>
+        <v>Sabotage: stewards catch a nobbler, chance (any planet without its own)</v>
       </c>
       <c r="B248">
-        <v>0.2</v>
+        <v>0.35</v>
+      </c>
+      <c r="C248" t="str">
+        <v>Rolled on race day from one draw per stable, made every week whether or not anybody booked a job, so the game stream never depends on a door</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>Sabotage: catch chance at Holy Bark</v>
+        <v>Sabotage: catch chance at Lagrange Lows</v>
       </c>
       <c r="B249">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v>Sabotage: caught, a flat fine</v>
+        <v>Sabotage: catch chance at Holy Bark</v>
       </c>
       <c r="B250">
-        <v>800</v>
-      </c>
-      <c r="C250" t="str">
-        <v>Paid as far as the cash goes: nobody is pushed into debt (V10)</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="str">
+        <v>Sabotage: caught, a flat fine</v>
+      </c>
+      <c r="B251">
+        <v>800</v>
+      </c>
+      <c r="C251" t="str">
+        <v>Paid as far as the cash goes: nobody is pushed into debt (V10)</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="str">
         <v>Sabotage: caught, share of what the nobbler had on the race</v>
       </c>
-      <c r="B251">
+      <c r="B252">
         <v>0.25</v>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" t="str">
-        <v>The game (GDD_V3 §2.1 — 1 to 5 seasons, or Race to a Target)</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="str">
-        <v>Game: fewest seasons a table may choose</v>
-      </c>
-      <c r="B254">
-        <v>1</v>
-      </c>
-      <c r="C254" t="str">
-        <v>The default game is one season, and a setup that names no length means one season</v>
+        <v>The game (GDD_V3 §2.1 — 1 to 5 seasons, or Race to a Target)</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>Game: most seasons a table may choose</v>
+        <v>Game: fewest seasons a table may choose</v>
       </c>
       <c r="B255">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="C255" t="str">
+        <v>The default game is one season, and a setup that names no length means one season</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>Target: suggested net worth, a short game</v>
+        <v>Game: most seasons a table may choose</v>
       </c>
       <c r="B256">
-        <v>60000</v>
-      </c>
-      <c r="C256" t="str">
-        <v>Net worth is checked at the end of every weekend; the first crossing ends the game at the end of that weekend, and the highest net worth wins (§2.1)</v>
+        <v>5</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>Target: suggested net worth, a long game</v>
+        <v>Target: suggested net worth, a short game</v>
       </c>
       <c r="B257">
-        <v>150000</v>
+        <v>60000</v>
+      </c>
+      <c r="C257" t="str">
+        <v>Net worth is checked at the end of every weekend; the first crossing ends the game at the end of that weekend, and the highest net worth wins (§2.1)</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="str">
+        <v>Target: suggested net worth, a long game</v>
+      </c>
+      <c r="B258">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="str">
         <v>Target: the most seasons a Target game runs</v>
       </c>
-      <c r="B258">
+      <c r="B259">
         <v>10</v>
       </c>
-      <c r="C258" t="str">
+      <c r="C259" t="str">
         <v>A cap so a target nobody reaches still ends. If it bites, the highest net worth wins as usual</v>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="str">
-        <v>The off-season (GDD_V3 §2.2 — age, one retirement, the staff notice)</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>Off-season: a trainer leaves, chance each</v>
-      </c>
-      <c r="B261">
-        <v>0.15</v>
-      </c>
-      <c r="C261" t="str">
-        <v>Rolled per trainer on the stable's own off-season stream. A stable left with fewer than two is offered one candidate</v>
+        <v>The off-season (GDD_V3 §2.2 — age, one retirement, the staff notice)</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>Off-season: the replacement's seller lies, × the dog-offer rate</v>
+        <v>Off-season: a trainer leaves, chance each</v>
       </c>
       <c r="B262">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="C262" t="str">
-        <v>A retirement is offered a replacement under §9.2: age, one true stat, and patter that lies at this × 0.35</v>
+        <v>Rolled per trainer on the stable's own off-season stream. A stable left with fewer than two is offered one candidate</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>Off-season: AI retires when the offer beats its cheapest dog by (Bones)</v>
+        <v>Off-season: the replacement's seller lies, × the dog-offer rate</v>
       </c>
       <c r="B263">
-        <v>500</v>
+        <v>1</v>
       </c>
       <c r="C263" t="str">
-        <v>Normal's rule: the offer as it can read it (estimateOffer) against the cheapest dog's book value plus this. Hard uses half</v>
+        <v>A retirement is offered a replacement under §9.2: age, one true stat, and patter that lies at this × 0.35</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>Off-season: AI retires a dog this old, whatever the offer</v>
+        <v>Off-season: AI retires when the offer beats its cheapest dog by (Bones)</v>
       </c>
       <c r="B264">
-        <v>6</v>
+        <v>500</v>
+      </c>
+      <c r="C264" t="str">
+        <v>Normal's rule: the offer as it can read it (estimateOffer) against the cheapest dog's book value plus this. Hard uses half</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
+        <v>Off-season: AI retires a dog this old, whatever the offer</v>
+      </c>
+      <c r="B265">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="str">
         <v>Off-season: every dog starts the new season on this fitness</v>
       </c>
-      <c r="B265">
+      <c r="B266">
         <v>100</v>
       </c>
-      <c r="C265" t="str">
+      <c r="C266" t="str">
         <v>Jesse's call for Phase E2: the off-season is a long rest. Any layoff clears too. Without it races entered fell from 2.12 a weekend in season 1 to about 1.87 after it</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D265"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D266"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add the draft's row to the sheet: the last stable's off-season offer, 15 above the ordinary
Jesse's pick from the Phase I sweep (GDD_V3 V23). add-phase-i-rows.ts
upserts one row under the off-season section; balance-from-xlsx.ts maps
it to draftLevelShift. Nothing reads it yet, so no golden moves here.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ABmefiezU3Mb4Bn9UsKLVH
</commit_message>
<xml_diff>
--- a/design/space_dog_racing_economy.xlsx
+++ b/design/space_dog_racing_economy.xlsx
@@ -526,7 +526,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D266"/>
+  <dimension ref="A1:D267"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2618,9 +2618,20 @@
         <v>Jesse's call for Phase E2: the off-season is a long rest. Any layoff clears too. Without it races entered fell from 2.12 a weekend in season 1 to about 1.87 after it</v>
       </c>
     </row>
+    <row r="267">
+      <c r="A267" t="str">
+        <v>Off-season: the draft, last stable's offer level above the ordinary (points)</v>
+      </c>
+      <c r="B267">
+        <v>15</v>
+      </c>
+      <c r="C267" t="str">
+        <v>Jesse's call for Phase I: the stable last on the season's standings is offered a better replacement dog, so a long game's back of the table can come back. Chosen from a sweep of 8 / 15 / 25 (and 15 for the bottom three) against a trailing stable arriving first and a bigger trainers' cut</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D266"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D267"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add the draft's rows to the sheet (Phase N, V29–V33)
Six new rows under a new section of the Assumptions sheet, through
add-phase-n-rows.ts (a copy of Phase I's upserter): the opening board's
dogs (5) and trainers (3) a stable, its rating range (40–60), the
off-season board's dogs a stable (1.5, rounded up) and the AI's
off-season margin (500 Bones). Nothing reads them yet, so nothing moves.

The rows this phase changes or retires (Starting dogs 4, the starting
crates, the dealt-dog and V23 rows) move with the engine in the next
commit, so this one stays green on its own.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0118hcT5DqA4T6PRGp8qULja
</commit_message>
<xml_diff>
--- a/design/space_dog_racing_economy.xlsx
+++ b/design/space_dog_racing_economy.xlsx
@@ -526,7 +526,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D267"/>
+  <dimension ref="A1:D275"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2629,9 +2629,77 @@
         <v>Jesse's call for Phase I: the stable last on the season's standings is offered a better replacement dog, so a long game's back of the table can come back. Chosen from a sweep of 8 / 15 / 25 (and 15 for the bottom three) against a trailing stable arriving first and a bigger trainers' cut</v>
       </c>
     </row>
+    <row r="269">
+      <c r="A269" t="str">
+        <v>The draft (GDD_V3 §2.2, §5.5 — four dogs and two trainers, picked from a board; V29–V33)</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="str">
+        <v>Draft: dogs on the opening board, per stable</v>
+      </c>
+      <c r="B270">
+        <v>5</v>
+      </c>
+      <c r="C270" t="str">
+        <v>V29/V31: the opening board carries this many dogs for every stable at the table; each stable drafts four, so a fifth of the board is left over</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="str">
+        <v>Draft: trainers on the opening board, per stable</v>
+      </c>
+      <c r="B271">
+        <v>3</v>
+      </c>
+      <c r="C271" t="str">
+        <v>V29: each stable drafts two; capped by the pool of 24, so eight stables see every trainer</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="str">
+        <v>Draft: the weakest dog on a board (rating)</v>
+      </c>
+      <c r="B272">
+        <v>40</v>
+      </c>
+      <c r="C272" t="str">
+        <v>V31: a board is rated evenly from this to the strongest, each style spanning the range, so a pick matters and the snake order keeps it fair</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="str">
+        <v>Draft: the strongest dog on a board (rating)</v>
+      </c>
+      <c r="B273">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="str">
+        <v>Draft: dogs on the off-season board, per stable (rounded up)</v>
+      </c>
+      <c r="B274">
+        <v>1.5</v>
+      </c>
+      <c r="C274" t="str">
+        <v>V32: one round, last on the standings picks first, from a fresh board of this many dogs a stable plus every unemployed trainer, up to one a stable</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="str">
+        <v>Draft: AI takes an off-season pick when it beats what it lets go by (Bones)</v>
+      </c>
+      <c r="B275">
+        <v>500</v>
+      </c>
+      <c r="C275" t="str">
+        <v>V32: otherwise it passes. Scored as book value plus expected season purses by rating (the harness fit)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D267"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D275"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Play the weekend at once, and give every stable three staff (Phase T)
Jesse's two calls (GDD_V3 T1-T4). Everybody plays the weekend at once: no
turn order is rolled, the door is the first thing in a stable's own weekend,
every stable has a shelf of its own (privateShelfShare of the posted depth),
and declarations are sealed until the last stable finishes - for an AI too
(sealedFor). A Mash glut or shortage is the finder's own price. Staff are a
Dog Trainer, a Trade Advisor and a Gambling Advisor, one of each, each paid a
share of their own side: purses, trading profit, winnings. The opening draft
is four dogs and one of each role. STATE_VERSION 16, PROTOCOL_VERSION 3.

The goldens move in the next commit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCVvvhvBJdSmAcRLngRmTS
</commit_message>
<xml_diff>
--- a/design/space_dog_racing_economy.xlsx
+++ b/design/space_dog_racing_economy.xlsx
@@ -526,7 +526,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D277"/>
+  <dimension ref="A1:D293"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2275,439 +2275,598 @@
     </row>
     <row r="228">
       <c r="A228" t="str">
-        <v>Staff: trainers dealt to each stable at the start of a game</v>
+        <v>Staff cut: +1 stat a week</v>
       </c>
       <c r="B228">
-        <v>2</v>
+        <v>0.03</v>
       </c>
       <c r="C228" t="str">
-        <v>Two slots, everyone a trainer (§8.1). Dealt at createSeason from the staff rows; the only way to change one in Phase D is a Bar card</v>
+        <v>Commission, a share of race prize money only (§8.1). A trainer with one bonus takes its cut; with two, the sum plus the premium below, capped</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
-        <v>Staff cut: +1 stat a week</v>
+        <v>Staff cut: +5 fitness recovery a week</v>
       </c>
       <c r="B229">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="C229" t="str">
-        <v>Commission, a share of race prize money only (§8.1). A trainer with one bonus takes its cut; with two, the sum plus the premium below, capped</v>
+        <v>3% at first. Measured at 800 seasons by regressing end worth on the dealt bonuses (the deal is random, so it is a clean experiment): a +5-recovery trainer was worth ~1,300 to its stable at 3%. 5% leaves it worth having</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
-        <v>Staff cut: +5 fitness recovery a week</v>
+        <v>Staff cut: injury chance halved</v>
       </c>
       <c r="B230">
-        <v>0.05</v>
-      </c>
-      <c r="C230" t="str">
-        <v>3% at first. Measured at 800 seasons by regressing end worth on the dealt bonuses (the deal is random, so it is a clean experiment): a +5-recovery trainer was worth ~1,300 to its stable at 3%. 5% leaves it worth having</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
-        <v>Staff cut: injury chance halved</v>
+        <v>Staff cut: injury duration −1 week</v>
       </c>
       <c r="B231">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
-        <v>Staff cut: injury duration −1 week</v>
+        <v>Gambling Advisor cut: a race-day tip a week, share of winnings</v>
       </c>
       <c r="B232">
-        <v>0.02</v>
+        <v>0.1</v>
+      </c>
+      <c r="C232" t="str">
+        <v>T4: was 2% of purses as a trainer bonus (Q3); a share of winnings now, and about rivals’ dogs only (a tip about your own dog is a Race-or-Rest call, the Trainer’s side). harness --draft, 17,000 stables (1,000 one-season games at 3, 6 and 8 stables, all Normal), Bones of end worth per bonus held net of its cut: at 10% and any dog +1,886 (± 511), fair 124%; at 30% and rivals only −161 (± 492), fair 20%; at 20% −153 (± 312) and −350 (± 315), fair −6 to 9%</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="str">
-        <v>Staff cut: a race-day tip a week</v>
+        <v>Trade Advisor cut: next week's prices for all six goods, share of trading profit</v>
       </c>
       <c r="B233">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="C233" t="str">
-        <v>Q3 (GDD_V3 §8.2, §14 Q13): the bonus that made a rival's style public became a race-day tip a week, since the draft (V30) made every drafted dog's style public; its 2% is unchanged. D12's regression on drafted trainers (17,000 stables, harness --draft): the style read at v3p −1,125 (± 439) Bones of end worth, a fair cut of −1.7%; the tip with Q1 and Q2 +278 (± 376), a fair cut of 2.9% (at 1%: +464 ± 325)</v>
+        <v>T4: was 8% of purses as a trainer bonus (D12’s regression); a share of trading profit now. harness --draft, 17,000 stables (1,000 one-season games at 3, 6 and 8 stables, all Normal), Bones of end worth per bonus held net of its cut: at 10% +823 (± 545), fair 26%; at 25% −800 (± 311), fair 8%; at 12% −662 (± 348) and −649 (± 375), fair below 0: Normal trades on a price it knows little better than on the map</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
-        <v>Staff cut: next planet's band position for all six goods</v>
+        <v>Staff cut: +10% prize money</v>
       </c>
       <c r="B234">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="C234" t="str">
-        <v>3% at first, and it was the cheapest bonus in the pool for what it did: knowing all six of next week's prices every week lifted food's share of gross income four points and was worth ~1,000 to its stable. At 8% the regression reads it at nothing either way — the same 8% trainer is cheap for a trader and dear for a racer (§8.1)</v>
+        <v>5% at first; 6% after the 800-season regression</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
-        <v>Staff cut: +10% prize money</v>
+        <v>Staff cut: Explore less likely to go badly</v>
       </c>
       <c r="B235">
-        <v>0.06</v>
-      </c>
-      <c r="C235" t="str">
-        <v>5% at first; 6% after the 800-season regression</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
-        <v>Staff cut: Explore less likely to go badly</v>
+        <v>Staff cut: premium for a trainer with two bonuses</v>
       </c>
       <c r="B236">
-        <v>0.03</v>
+        <v>0.02</v>
+      </c>
+      <c r="C236" t="str">
+        <v>§8.2: "two of the above, 6–10%". The cheapest pair (2% + 2%) lands on 6%</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
-        <v>Staff cut: premium for a trainer with two bonuses</v>
+        <v>Staff cut: the most a trainer takes</v>
       </c>
       <c r="B237">
-        <v>0.02</v>
+        <v>0.1</v>
       </c>
       <c r="C237" t="str">
-        <v>§8.2: "two of the above, 6–10%". The cheapest pair (2% + 2%) lands on 6%</v>
+        <v>§8.1: 1–10%. A 10% trainer on a stable earning 30,000 in purses costs 3,000</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
-        <v>Staff cut: the most a trainer takes</v>
+        <v>Staff bonus: fitness a week, to a dog that did not run</v>
       </c>
       <c r="B238">
-        <v>0.1</v>
+        <v>5</v>
       </c>
       <c r="C238" t="str">
-        <v>§8.1: 1–10%. A 10% trainer on a stable earning 30,000 in purses costs 3,000</v>
+        <v>Folded into weeklyFitnessDelta's bonus, so it goes through the week's one clamp</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
-        <v>Staff bonus: fitness a week, to a dog that did not run</v>
+        <v>Staff bonus: injury chance ×</v>
       </c>
       <c r="B239">
-        <v>5</v>
-      </c>
-      <c r="C239" t="str">
-        <v>Folded into weeklyFitnessDelta's bonus, so it goes through the week's one clamp</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
-        <v>Staff bonus: injury chance ×</v>
+        <v>Staff bonus: weeks off a layoff, at the roll</v>
       </c>
       <c r="B240">
-        <v>0.5</v>
+        <v>1</v>
+      </c>
+      <c r="C240" t="str">
+        <v>Never below one week</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
-        <v>Staff bonus: weeks off a layoff, at the roll</v>
+        <v>Staff bonus: extra prize money, share of the purse</v>
       </c>
       <c r="B241">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="C241" t="str">
-        <v>Never below one week</v>
+        <v>Added before the commission is taken</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
-        <v>Staff bonus: extra prize money, share of the purse</v>
+        <v>Staff bonus: an Explore card's bad-outcome chance ×</v>
       </c>
       <c r="B242">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="C242" t="str">
-        <v>Added before the commission is taken</v>
+        <v>Read by every card through the kit's risk() and luck() helpers, never by a branch</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
-        <v>Staff bonus: an Explore card's bad-outcome chance ×</v>
+        <v>Staff bonus: stat points a week, to one dog</v>
       </c>
       <c r="B243">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="C243" t="str">
-        <v>Read by every card through the kit's risk() and luck() helpers, never by a branch</v>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" t="str">
-        <v>Staff bonus: stat points a week, to one dog</v>
-      </c>
-      <c r="B244">
-        <v>1</v>
-      </c>
-      <c r="C244" t="str">
         <v>§8.2's "+1 to one stat per week": at the jump, beside the food, on the lowest-rated dog's weakest stat by the rating's weights — a rule, not a draw. Built first as +1 to every dog, which made a 3% trainer worth ~4,000 of end worth and took mean end worth out of its band (decision D10)</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v>Sabotage (GDD_V3 §9.3 — a nobble, a bought box, and the stewards who might notice)</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>Sabotage (GDD_V3 §9.3 — a nobble, a bought box, and the stewards who might notice)</v>
+        <v>Sabotage: a nobbled runner's fitness on race day</v>
+      </c>
+      <c r="B246">
+        <v>-25</v>
+      </c>
+      <c r="C246" t="str">
+        <v>Applied to the runner, like a race-day condition: the book has struck its prices and the victim's stated fitness never changes</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>Sabotage: a nobbled runner's fitness on race day</v>
+        <v>Sabotage: stewards catch a nobbler, chance (any planet without its own)</v>
       </c>
       <c r="B247">
-        <v>-25</v>
+        <v>0.35</v>
       </c>
       <c r="C247" t="str">
-        <v>Applied to the runner, like a race-day condition: the book has struck its prices and the victim's stated fitness never changes</v>
+        <v>Rolled on race day from one draw per stable, made every week whether or not anybody booked a job, so the game stream never depends on a door</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>Sabotage: stewards catch a nobbler, chance (any planet without its own)</v>
+        <v>Sabotage: catch chance at Lagrange Lows</v>
       </c>
       <c r="B248">
-        <v>0.35</v>
-      </c>
-      <c r="C248" t="str">
-        <v>Rolled on race day from one draw per stable, made every week whether or not anybody booked a job, so the game stream never depends on a door</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>Sabotage: catch chance at Lagrange Lows</v>
+        <v>Sabotage: catch chance at Holy Bark</v>
       </c>
       <c r="B249">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v>Sabotage: catch chance at Holy Bark</v>
+        <v>Sabotage: caught, a flat fine</v>
       </c>
       <c r="B250">
-        <v>0.6</v>
+        <v>800</v>
+      </c>
+      <c r="C250" t="str">
+        <v>Paid as far as the cash goes: nobody is pushed into debt (V10)</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="str">
-        <v>Sabotage: caught, a flat fine</v>
+        <v>Sabotage: caught, share of what the nobbler had on the race</v>
       </c>
       <c r="B251">
-        <v>800</v>
-      </c>
-      <c r="C251" t="str">
-        <v>Paid as far as the cash goes: nobody is pushed into debt (V10)</v>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="str">
-        <v>Sabotage: caught, share of what the nobbler had on the race</v>
-      </c>
-      <c r="B252">
         <v>0.25</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="str">
+        <v>The game (GDD_V3 §2.1 — 1 to 5 seasons, or Race to a Target)</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="str">
-        <v>The game (GDD_V3 §2.1 — 1 to 5 seasons, or Race to a Target)</v>
+        <v>Game: fewest seasons a table may choose</v>
+      </c>
+      <c r="B254">
+        <v>1</v>
+      </c>
+      <c r="C254" t="str">
+        <v>The default game is one season, and a setup that names no length means one season</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>Game: fewest seasons a table may choose</v>
+        <v>Game: most seasons a table may choose</v>
       </c>
       <c r="B255">
-        <v>1</v>
-      </c>
-      <c r="C255" t="str">
-        <v>The default game is one season, and a setup that names no length means one season</v>
+        <v>5</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>Game: most seasons a table may choose</v>
+        <v>Target: suggested net worth, a short game</v>
       </c>
       <c r="B256">
-        <v>5</v>
+        <v>60000</v>
+      </c>
+      <c r="C256" t="str">
+        <v>Net worth is checked at the end of every weekend; the first crossing ends the game at the end of that weekend, and the highest net worth wins (§2.1)</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>Target: suggested net worth, a short game</v>
+        <v>Target: suggested net worth, a long game</v>
       </c>
       <c r="B257">
-        <v>60000</v>
-      </c>
-      <c r="C257" t="str">
-        <v>Net worth is checked at the end of every weekend; the first crossing ends the game at the end of that weekend, and the highest net worth wins (§2.1)</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>Target: suggested net worth, a long game</v>
+        <v>Target: the most seasons a Target game runs</v>
       </c>
       <c r="B258">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" t="str">
-        <v>Target: the most seasons a Target game runs</v>
-      </c>
-      <c r="B259">
         <v>10</v>
       </c>
-      <c r="C259" t="str">
+      <c r="C258" t="str">
         <v>A cap so a target nobody reaches still ends. If it bites, the highest net worth wins as usual</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>The off-season (GDD_V3 §2.2 — age, one retirement, the staff notice)</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>The off-season (GDD_V3 §2.2 — age, one retirement, the staff notice)</v>
+        <v>Off-season: a member of staff leaves, chance each</v>
+      </c>
+      <c r="B261">
+        <v>0.15</v>
+      </c>
+      <c r="C261" t="str">
+        <v>E5, unchanged: every member of staff, of every role, rolls it</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>Off-season: a trainer leaves, chance each</v>
+        <v>Off-season: every dog starts the new season on this fitness</v>
       </c>
       <c r="B262">
-        <v>0.15</v>
+        <v>100</v>
       </c>
       <c r="C262" t="str">
-        <v>Rolled per trainer on the stable's own off-season stream. A stable left with fewer than two is offered one candidate</v>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" t="str">
-        <v>Off-season: every dog starts the new season on this fitness</v>
-      </c>
-      <c r="B263">
-        <v>100</v>
-      </c>
-      <c r="C263" t="str">
         <v>Jesse's call for Phase E2: the off-season is a long rest. Any layoff clears too. Without it races entered fell from 2.12 a weekend in season 1 to about 1.87 after it</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>The draft (GDD_V3 §2.2, §5.5 — four dogs and two trainers, picked from a board; V29–V33)</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>The draft (GDD_V3 §2.2, §5.5 — four dogs and two trainers, picked from a board; V29–V33)</v>
+        <v>Draft: dogs on the opening board, per stable</v>
+      </c>
+      <c r="B265">
+        <v>5</v>
+      </c>
+      <c r="C265" t="str">
+        <v>V29/V31: the opening board carries this many dogs for every stable at the table; each stable drafts four, so a fifth of the board is left over</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>Draft: dogs on the opening board, per stable</v>
+        <v>Draft: staff of each role on the opening board, per stable (rounded up)</v>
       </c>
       <c r="B266">
-        <v>5</v>
+        <v>1.5</v>
       </c>
       <c r="C266" t="str">
-        <v>V29/V31: the opening board carries this many dogs for every stable at the table; each stable drafts four, so a fifth of the board is left over</v>
+        <v>T2: the opening draft takes one of each role, so the board carries 1.5 a stable of each — the 1.5× choice the two-trainer board gave (3 a stable for 2 picks). 12 of each at 8 stables, which is every Trade and Gambling Advisor there is</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>Draft: trainers on the opening board, per stable</v>
+        <v>Draft: the weakest dog on a board (rating)</v>
       </c>
       <c r="B267">
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="C267" t="str">
-        <v>V29: each stable drafts two; capped by the pool of 24, so eight stables see every trainer</v>
+        <v>V31: the opening board is rated evenly from this to the strongest, each style spanning the range, so a pick matters and the snake order keeps it fair. 40–60 until Jesse's call at Phase N (45–55), which narrowed the first pick's edge at eight stables</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="str">
-        <v>Draft: the weakest dog on a board (rating)</v>
+        <v>Draft: the strongest dog on a board (rating)</v>
       </c>
       <c r="B268">
-        <v>45</v>
-      </c>
-      <c r="C268" t="str">
-        <v>V31: the opening board is rated evenly from this to the strongest, each style spanning the range, so a pick matters and the snake order keeps it fair. 40–60 until Jesse's call at Phase N (45–55), which narrowed the first pick's edge at eight stables</v>
+        <v>55</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="str">
-        <v>Draft: the strongest dog on a board (rating)</v>
+        <v>Draft: dogs on the off-season board, per stable (rounded up)</v>
       </c>
       <c r="B269">
-        <v>55</v>
+        <v>1</v>
+      </c>
+      <c r="C269" t="str">
+        <v>V32: one round, last on the standings picks first, from a fresh board of this many dogs a stable plus every unemployed trainer, up to one a stable. 1.5 as first built; Jesse's call at Phase N was one, so the leader's pick is the board's worst dog</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="str">
-        <v>Draft: dogs on the off-season board, per stable (rounded up)</v>
+        <v>Draft: AI takes an off-season pick when it beats what it lets go by (Bones)</v>
       </c>
       <c r="B270">
-        <v>1</v>
+        <v>500</v>
       </c>
       <c r="C270" t="str">
-        <v>V32: one round, last on the standings picks first, from a fresh board of this many dogs a stable plus every unemployed trainer, up to one a stable. 1.5 as first built; Jesse's call at Phase N was one, so the leader's pick is the board's worst dog</v>
+        <v>V32: otherwise it passes. Scored as book value plus expected season purses by rating (the harness fit)</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="str">
-        <v>Draft: AI takes an off-season pick when it beats what it lets go by (Bones)</v>
+        <v>Draft: the weakest dog on the off-season board (rating)</v>
       </c>
       <c r="B271">
-        <v>500</v>
+        <v>40</v>
       </c>
       <c r="C271" t="str">
-        <v>V32: otherwise it passes. Scored as book value plus expected season purses by rating (the harness fit)</v>
+        <v>V32: the off-season board's own range, so the opening board can be narrowed without taking the back of the table's catch-up with it</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="str">
-        <v>Draft: the weakest dog on the off-season board (rating)</v>
+        <v>Draft: the strongest dog on the off-season board (rating)</v>
       </c>
       <c r="B272">
-        <v>40</v>
-      </c>
-      <c r="C272" t="str">
-        <v>V32: the off-season board's own range, so the opening board can be narrowed without taking the back of the table's catch-up with it</v>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" t="str">
-        <v>Draft: the strongest dog on the off-season board (rating)</v>
-      </c>
-      <c r="B273">
         <v>60</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="str">
+        <v>Phase Q (v3q) — Claude's unattended changes, each a Q row in GDD_V3 §13</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="str">
-        <v>Phase Q (v3q) — Claude's unattended changes, each a Q row in GDD_V3 §13</v>
+        <v>Book: rating points a fitness point is worth, against a local at 75</v>
+      </c>
+      <c r="B275">
+        <v>0.2</v>
+      </c>
+      <c r="C275" t="str">
+        <v>Q1 (GDD_V3 §5.6, §14 Q9): the book prices a stable runner's fitness, rounded to whole rating points; locals are always priced at 75. At 0 (v3p) a 1-Bone win bet on a stable runner at fitness 100 returned +92%, at 80–89 +22%, under 60 −33%; at 0.1 +35% / +9% / −22%; at 0.2 +8% / +3% / −7%; at 0.3 −15% / −3% / +16%</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>Book: rating points a fitness point is worth, against a local at 75</v>
+        <v>Draft: round 3 runs the way round 2 did (1 yes, 0 a plain snake)</v>
       </c>
       <c r="B276">
+        <v>1</v>
+      </c>
+      <c r="C276" t="str">
+        <v>Q2 (GDD_V3 §5.5, V29): the third-round reversal. Win rate by draft position, widest gap from fair at 3 / 6 / 8 stables, all Normal, one season: plain snake 4.4 / 5.2 / 4.7 points (1,000 games); round 3 reversed 1.0 / 2.0 / 3.1 (1,000) and 2.3 / 1.1 / 2.7 (2,000) against ±3. Jesse's 45–55 board is untouched. Phase T (seven rounds: four dogs, then one of each staff role), 1,000 games, with the staff priced as they ship: reversed 1.7 / 1.8 / 2.2, MET; plain snake 4.0 / 4.7 / 6.8, the first pick taking the first Trainer. Kept on</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="str">
+        <v>Phase T (v3t) — the weekend at once, and three staff (GDD_V3 T1–T4)</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="str">
+        <v>Trade Advisor bonus: every crate bought costs this share less</v>
+      </c>
+      <c r="B279">
+        <v>0.05</v>
+      </c>
+      <c r="C279" t="str">
+        <v>T3 [estimate]. With the sell price raised by sellUp it must stay under foodSpread (0.10) or a crate bought and sold in one place would pay; the engine also holds a stable’s sell price under its buy price</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="str">
+        <v>Trade Advisor bonus: every crate sold fetches this share more</v>
+      </c>
+      <c r="B280">
+        <v>0.04</v>
+      </c>
+      <c r="C280" t="str">
+        <v>T3 [estimate]</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="str">
+        <v>Trade Advisor bonus: the stable’s own shelf is this share deeper</v>
+      </c>
+      <c r="B281">
+        <v>0.25</v>
+      </c>
+      <c r="C281" t="str">
+        <v>T3. Rounded up per good. Measured at 0.5 by harness --draft (17,000 stables): +1,941 (± 279) of end worth, a fair cut of 43% of trading profit; halved, and its cut raised</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="str">
+        <v>Gambling Advisor bonus: a slip’s odds are this share better</v>
+      </c>
+      <c r="B282">
+        <v>0.05</v>
+      </c>
+      <c r="C282" t="str">
+        <v>T3. At the 15% margin a blind slip returns 0.85 × 1.05 = 0.89 a Bone: still a loss without a read. At 0.08: +733 (± 358), a fair cut of 56% of winnings; cut back to 0.05</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="str">
+        <v>Gambling Advisor bonus: the flat stake ceiling is this share higher</v>
+      </c>
+      <c r="B283">
+        <v>0.5</v>
+      </c>
+      <c r="C283" t="str">
+        <v>T3 [estimate]. 1,000 → 1,500 a race (Neon Snout 3,000); the share-of-cash fraction is unchanged</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="str">
+        <v>Trade Advisor cut: buys cheaper, share of trading profit</v>
+      </c>
+      <c r="B284">
         <v>0.2</v>
       </c>
-      <c r="C276" t="str">
-        <v>Q1 (GDD_V3 §5.6, §14 Q9): the book prices a stable runner's fitness, rounded to whole rating points; locals are always priced at 75. At 0 (v3p) a 1-Bone win bet on a stable runner at fitness 100 returned +92%, at 80–89 +22%, under 60 −33%; at 0.1 +35% / +9% / −22%; at 0.2 +8% / +3% / −7%; at 0.3 −15% / −3% / +16%</v>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" t="str">
-        <v>Draft: round 3 runs the way round 2 did (1 yes, 0 a plain snake)</v>
-      </c>
-      <c r="B277">
-        <v>1</v>
-      </c>
-      <c r="C277" t="str">
-        <v>Q2 (GDD_V3 §5.5, V29): the third-round reversal. Win rate by draft position, widest gap from fair at 3 / 6 / 8 stables, all Normal, one season: plain snake 4.4 / 5.2 / 4.7 points (1,000 games); round 3 reversed 1.0 / 2.0 / 3.1 (1,000) and 2.3 / 1.1 / 2.7 (2,000) against ±3. Jesse's 45–55 board is untouched</v>
+      <c r="C284" t="str">
+        <v>T4. Trading profit is (sell − You Paid) × crates on every sale that makes one, about 4,800 a stable-season. harness --draft, 17,000 stables (1,000 one-season games at 3, 6 and 8 stables, all Normal), Bones of end worth per bonus held net of its cut: at 8% +741 (± 438), fair 22%; at 20% +229 (± 299), fair 25%; at 22% −179 (± 244) and +65 (± 241), fair 18–23%</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="str">
+        <v>Trade Advisor cut: sells dearer, share of trading profit</v>
+      </c>
+      <c r="B285">
+        <v>0.03</v>
+      </c>
+      <c r="C285" t="str">
+        <v>T4. harness --draft, 17,000 stables (1,000 one-season games at 3, 6 and 8 stables, all Normal), Bones of end worth per bonus held net of its cut: at 8% +62 (± 329), fair 9%; again at 8% −244 (± 391), fair 3%; at 5% −384 (± 290) and −126 (± 278), fair 2–3%</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="str">
+        <v>Trade Advisor cut: a deeper shelf, share of trading profit</v>
+      </c>
+      <c r="B286">
+        <v>0.15</v>
+      </c>
+      <c r="C286" t="str">
+        <v>T4. harness --draft, 17,000 stables (1,000 one-season games at 3, 6 and 8 stables, all Normal), Bones of end worth per bonus held net of its cut: at 6% with a +50% shelf +1,941 (± 279), fair 43%; at 20% with +25% +147 (± 276), fair 23%; at 22% −245 (± 261) and −437 (± 265), fair 13–17%</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="str">
+        <v>Gambling Advisor cut: better odds, share of winnings</v>
+      </c>
+      <c r="B287">
+        <v>0.15</v>
+      </c>
+      <c r="C287" t="str">
+        <v>T4. Winnings are payout − stake on every slip that wins, about 1,500 a stable-season. harness --draft, 17,000 stables (1,000 one-season games at 3, 6 and 8 stables, all Normal), Bones of end worth per bonus held net of its cut: at 12% with +8% odds +733 (± 358), fair 56%; at 30% with +5% −75 (± 311), fair 25%; at 25% −428 (± 309) and −384 (± 314), fair below 0 — noisy: winnings are a small side, and Normal bets little</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="str">
+        <v>Gambling Advisor cut: a higher stake ceiling, share of winnings</v>
+      </c>
+      <c r="B288">
+        <v>0.02</v>
+      </c>
+      <c r="C288" t="str">
+        <v>T4. harness --draft, 17,000 stables (1,000 one-season games at 3, 6 and 8 stables, all Normal), Bones of end worth per bonus held net of its cut: at 8% +108 (± 265), fair 14.5%; at 12% −343 (± 283), fair below zero: Normal seldom bets at the ceiling, so the lift is worth little to it. Held at the floor of the 1–10% range rather than given away; at 5% −406 (± 441) and −475 (± 427): held near nothing</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="str">
+        <v>Staff cut: the most an advisor takes, of their side</v>
+      </c>
+      <c r="B289">
+        <v>0.4</v>
+      </c>
+      <c r="C289" t="str">
+        <v>T4: a Trainer is still capped at staffCutMax (10% of purses); an advisor’s side is a profit, a fifth of the purses (trade) or a seventeenth (winnings), so its cap is higher</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="str">
+        <v>Arrival: fitness a rested landing gives (a wormhole, a pilot’s chart)</v>
+      </c>
+      <c r="B290">
+        <v>10</v>
+      </c>
+      <c r="C290" t="str">
+        <v>T1: the two cards that bought "arrive first next week" — there is no turn order to be first in</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="str">
+        <v>Arrival: fitness a shaken landing costs (a fried navicomp)</v>
+      </c>
+      <c r="B291">
+        <v>-10</v>
+      </c>
+      <c r="C291" t="str">
+        <v>T1: the Solar flare card’s "land last next week"</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="str">
+        <v>Blackreach: every stable’s shelf is this many times the posted depth</v>
+      </c>
+      <c r="B292">
+        <v>2</v>
+      </c>
+      <c r="C292" t="str">
+        <v>T1: Blackreach reversed the turn order; with no turn order its time-bending station restocks twice</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="str">
+        <v>Market: a stable’s own shelf is this share of the posted depth (rounded up)</v>
+      </c>
+      <c r="B293">
+        <v>0.2</v>
+      </c>
+      <c r="C293" t="str">
+        <v>T2: every stable has a shelf of its own now. The posted depths (the goods rows above) were a whole table’s shelf, shared in turn order; given whole to every stable they tripled the trade (food sold 10,399 → 34,737 gross a stable-season, cash-bound → hold-bound at week 1.9). Six Normal stables, 50 seasons: at 0.15 food sold 10,313, crossover week 5.1 (19% of stable-seasons cross); at 0.2 13,417, week 4.7 (45%); at 0.25 15,489; at 0.3 18,500. v3s: 10,399, week 4.6 (73%). 0.2 is the nearest to v3s on the crossover row, which is the progression §6.1 is about</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D277"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D293"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>